<commit_message>
ajouts de réalisations pro
</commit_message>
<xml_diff>
--- a/docs/SSZ_TableauDeSynthese.xlsx
+++ b/docs/SSZ_TableauDeSynthese.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="46">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -170,9 +170,6 @@
     <t>Stage dans l'entreprise Prakti.net</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>Projet 1 : landing pagede prakti.net</t>
   </si>
   <si>
@@ -184,7 +181,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -195,14 +192,35 @@
     <font>
       <b/>
       <sz val="20"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="18"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -213,49 +231,34 @@
       <family val="2"/>
     </font>
     <font>
-      <b/>
-      <i/>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="10"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="14"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="16"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="8"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -661,10 +664,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="49">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
@@ -729,8 +735,8 @@
     <xf xfId="0" numFmtId="0" borderId="18" applyBorder="1" fontId="5" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="6" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="19" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -738,71 +744,71 @@
     <xf xfId="0" numFmtId="0" borderId="20" applyBorder="1" fontId="5" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="21" applyBorder="1" fontId="6" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="21" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="22" applyBorder="1" fontId="6" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="22" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="23" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="23" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="17" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="17" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="18" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="18" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="24" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="24" applyBorder="1" fontId="9" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="25" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="25" applyBorder="1" fontId="9" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="25" applyBorder="1" fontId="9" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="25" applyBorder="1" fontId="10" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="26" applyBorder="1" fontId="10" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="25" applyBorder="1" fontId="11" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="24" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="26" applyBorder="1" fontId="11" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="25" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="24" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="26" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="25" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="25" applyBorder="1" fontId="10" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="26" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="27" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="27" applyBorder="1" fontId="9" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="28" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="28" applyBorder="1" fontId="9" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="28" applyBorder="1" fontId="10" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="28" applyBorder="1" fontId="11" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="29" applyBorder="1" fontId="10" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="29" applyBorder="1" fontId="11" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="9" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="9" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="10" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="11" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1117,44 +1123,44 @@
     <col min="6" max="6" style="47" width="18.719285714285714" customWidth="1" bestFit="1"/>
     <col min="7" max="7" style="47" width="18.719285714285714" customWidth="1" bestFit="1"/>
     <col min="8" max="8" style="47" width="18.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="47" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="47" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
     <col min="11" max="11" style="47" width="11.43357142857143" customWidth="1" bestFit="1"/>
     <col min="12" max="12" style="47" width="11.43357142857143" customWidth="1" bestFit="1"/>
     <col min="13" max="13" style="47" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="47" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="47" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="47" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="47" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="47" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="47" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="47" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="47" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="47" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="23" max="23" style="47" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="24" max="24" style="47" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="25" max="25" style="47" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="26" max="26" style="47" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="27" max="27" style="47" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="28" max="28" style="47" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="29" max="29" style="47" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="30" max="30" style="47" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="31" max="31" style="47" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="32" max="32" style="47" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="33" max="33" style="47" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="34" max="34" style="47" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="35" max="35" style="47" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="36" max="36" style="47" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="37" max="37" style="47" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="38" max="38" style="47" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="39" max="39" style="47" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="40" max="40" style="47" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="41" max="41" style="47" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="42" max="42" style="47" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="43" max="43" style="47" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="23" max="23" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="24" max="24" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="25" max="25" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="26" max="26" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="27" max="27" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="28" max="28" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="29" max="29" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="30" max="30" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="31" max="31" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="32" max="32" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="33" max="33" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="34" max="34" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="35" max="35" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="36" max="36" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="37" max="37" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="38" max="38" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="39" max="39" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="40" max="40" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="41" max="41" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="42" max="42" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="43" max="43" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="39.95">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="29.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1169,9 +1175,9 @@
       <c r="H1" s="1"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
-      <c r="M1" s="2"/>
+      <c r="K1" s="3"/>
+      <c r="L1" s="3"/>
+      <c r="M1" s="3"/>
       <c r="N1" s="2"/>
       <c r="O1" s="2"/>
       <c r="P1" s="2"/>
@@ -1203,7 +1209,7 @@
       <c r="AP1" s="2"/>
       <c r="AQ1" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="41.1">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="29.25">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -1216,9 +1222,9 @@
       <c r="H2" s="1"/>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
-      <c r="M2" s="2"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
       <c r="N2" s="2"/>
       <c r="O2" s="2"/>
       <c r="P2" s="2"/>
@@ -1250,24 +1256,24 @@
       <c r="AP2" s="2"/>
       <c r="AQ2" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="39.95">
-      <c r="A3" s="3" t="s">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="27">
+      <c r="A3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="6" t="s">
+      <c r="B3" s="5"/>
+      <c r="C3" s="5"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="4"/>
-      <c r="H3" s="7"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="8"/>
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
-      <c r="K3" s="8"/>
-      <c r="L3" s="8"/>
-      <c r="M3" s="8"/>
+      <c r="K3" s="9"/>
+      <c r="L3" s="9"/>
+      <c r="M3" s="9"/>
       <c r="N3" s="2"/>
       <c r="O3" s="2"/>
       <c r="P3" s="2"/>
@@ -1299,28 +1305,28 @@
       <c r="AP3" s="2"/>
       <c r="AQ3" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="39.95">
-      <c r="A4" s="9" t="s">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="27.75">
+      <c r="A4" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="10"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="12" t="s">
+      <c r="B4" s="11"/>
+      <c r="C4" s="11"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="G4" s="13" t="s">
+      <c r="G4" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="H4" s="14" t="s">
+      <c r="H4" s="15" t="s">
         <v>8</v>
       </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
-      <c r="M4" s="2"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+      <c r="M4" s="3"/>
       <c r="N4" s="2"/>
       <c r="O4" s="2"/>
       <c r="P4" s="2"/>
@@ -1352,22 +1358,22 @@
       <c r="AP4" s="2"/>
       <c r="AQ4" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="39.95">
-      <c r="A5" s="15" t="s">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="27.75">
+      <c r="A5" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="16"/>
-      <c r="C5" s="16"/>
-      <c r="D5" s="16"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="16"/>
-      <c r="G5" s="16"/>
-      <c r="H5" s="17"/>
+      <c r="B5" s="17"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="17"/>
+      <c r="F5" s="17"/>
+      <c r="G5" s="17"/>
+      <c r="H5" s="18"/>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
-      <c r="L5" s="2"/>
-      <c r="M5" s="2"/>
+      <c r="K5" s="3"/>
+      <c r="L5" s="3"/>
+      <c r="M5" s="3"/>
       <c r="N5" s="2"/>
       <c r="O5" s="2"/>
       <c r="P5" s="2"/>
@@ -1399,140 +1405,140 @@
       <c r="AP5" s="2"/>
       <c r="AQ5" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="90" customFormat="1" s="18">
-      <c r="A6" s="19" t="s">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="165.375" customFormat="1" s="19">
+      <c r="A6" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="20" t="s">
+      <c r="B6" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="21" t="s">
+      <c r="C6" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="21" t="s">
+      <c r="D6" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="21" t="s">
+      <c r="E6" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="F6" s="21" t="s">
+      <c r="F6" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="G6" s="21" t="s">
+      <c r="G6" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="H6" s="22" t="s">
+      <c r="H6" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="I6" s="23"/>
-      <c r="J6" s="23"/>
-      <c r="K6" s="23"/>
-      <c r="L6" s="23"/>
-      <c r="M6" s="23"/>
-      <c r="N6" s="23"/>
-      <c r="O6" s="23"/>
-      <c r="P6" s="23"/>
-      <c r="Q6" s="23"/>
-      <c r="R6" s="23"/>
-      <c r="S6" s="23"/>
-      <c r="T6" s="23"/>
-      <c r="U6" s="23"/>
-      <c r="V6" s="23"/>
-      <c r="W6" s="23"/>
-      <c r="X6" s="23"/>
-      <c r="Y6" s="23"/>
-      <c r="Z6" s="23"/>
-      <c r="AA6" s="23"/>
-      <c r="AB6" s="23"/>
-      <c r="AC6" s="23"/>
-      <c r="AD6" s="23"/>
-      <c r="AE6" s="23"/>
-      <c r="AF6" s="23"/>
-      <c r="AG6" s="23"/>
-      <c r="AH6" s="23"/>
-      <c r="AI6" s="23"/>
-      <c r="AJ6" s="23"/>
-      <c r="AK6" s="23"/>
-      <c r="AL6" s="23"/>
-      <c r="AM6" s="23"/>
-      <c r="AN6" s="23"/>
-      <c r="AO6" s="23"/>
-      <c r="AP6" s="23"/>
-      <c r="AQ6" s="23"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="292.5" customFormat="1" s="18">
-      <c r="A7" s="24"/>
-      <c r="B7" s="25"/>
-      <c r="C7" s="26" t="s">
+      <c r="I6" s="24"/>
+      <c r="J6" s="24"/>
+      <c r="K6" s="24"/>
+      <c r="L6" s="24"/>
+      <c r="M6" s="24"/>
+      <c r="N6" s="24"/>
+      <c r="O6" s="24"/>
+      <c r="P6" s="24"/>
+      <c r="Q6" s="24"/>
+      <c r="R6" s="24"/>
+      <c r="S6" s="24"/>
+      <c r="T6" s="24"/>
+      <c r="U6" s="24"/>
+      <c r="V6" s="24"/>
+      <c r="W6" s="24"/>
+      <c r="X6" s="24"/>
+      <c r="Y6" s="24"/>
+      <c r="Z6" s="24"/>
+      <c r="AA6" s="24"/>
+      <c r="AB6" s="24"/>
+      <c r="AC6" s="24"/>
+      <c r="AD6" s="24"/>
+      <c r="AE6" s="24"/>
+      <c r="AF6" s="24"/>
+      <c r="AG6" s="24"/>
+      <c r="AH6" s="24"/>
+      <c r="AI6" s="24"/>
+      <c r="AJ6" s="24"/>
+      <c r="AK6" s="24"/>
+      <c r="AL6" s="24"/>
+      <c r="AM6" s="24"/>
+      <c r="AN6" s="24"/>
+      <c r="AO6" s="24"/>
+      <c r="AP6" s="24"/>
+      <c r="AQ6" s="24"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="292.5" customFormat="1" s="19">
+      <c r="A7" s="25"/>
+      <c r="B7" s="26"/>
+      <c r="C7" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="26" t="s">
+      <c r="D7" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="E7" s="26" t="s">
+      <c r="E7" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="F7" s="26" t="s">
+      <c r="F7" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="G7" s="26" t="s">
+      <c r="G7" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="H7" s="27" t="s">
+      <c r="H7" s="28" t="s">
         <v>23</v>
       </c>
-      <c r="I7" s="23"/>
-      <c r="J7" s="23"/>
-      <c r="K7" s="23"/>
-      <c r="L7" s="23"/>
-      <c r="M7" s="23"/>
-      <c r="N7" s="23"/>
-      <c r="O7" s="23"/>
-      <c r="P7" s="23"/>
-      <c r="Q7" s="23"/>
-      <c r="R7" s="23"/>
-      <c r="S7" s="23"/>
-      <c r="T7" s="23"/>
-      <c r="U7" s="23"/>
-      <c r="V7" s="23"/>
-      <c r="W7" s="23"/>
-      <c r="X7" s="23"/>
-      <c r="Y7" s="23"/>
-      <c r="Z7" s="23"/>
-      <c r="AA7" s="23"/>
-      <c r="AB7" s="23"/>
-      <c r="AC7" s="23"/>
-      <c r="AD7" s="23"/>
-      <c r="AE7" s="23"/>
-      <c r="AF7" s="23"/>
-      <c r="AG7" s="23"/>
-      <c r="AH7" s="23"/>
-      <c r="AI7" s="23"/>
-      <c r="AJ7" s="23"/>
-      <c r="AK7" s="23"/>
-      <c r="AL7" s="23"/>
-      <c r="AM7" s="23"/>
-      <c r="AN7" s="23"/>
-      <c r="AO7" s="23"/>
-      <c r="AP7" s="23"/>
-      <c r="AQ7" s="23"/>
+      <c r="I7" s="24"/>
+      <c r="J7" s="24"/>
+      <c r="K7" s="24"/>
+      <c r="L7" s="24"/>
+      <c r="M7" s="24"/>
+      <c r="N7" s="24"/>
+      <c r="O7" s="24"/>
+      <c r="P7" s="24"/>
+      <c r="Q7" s="24"/>
+      <c r="R7" s="24"/>
+      <c r="S7" s="24"/>
+      <c r="T7" s="24"/>
+      <c r="U7" s="24"/>
+      <c r="V7" s="24"/>
+      <c r="W7" s="24"/>
+      <c r="X7" s="24"/>
+      <c r="Y7" s="24"/>
+      <c r="Z7" s="24"/>
+      <c r="AA7" s="24"/>
+      <c r="AB7" s="24"/>
+      <c r="AC7" s="24"/>
+      <c r="AD7" s="24"/>
+      <c r="AE7" s="24"/>
+      <c r="AF7" s="24"/>
+      <c r="AG7" s="24"/>
+      <c r="AH7" s="24"/>
+      <c r="AI7" s="24"/>
+      <c r="AJ7" s="24"/>
+      <c r="AK7" s="24"/>
+      <c r="AL7" s="24"/>
+      <c r="AM7" s="24"/>
+      <c r="AN7" s="24"/>
+      <c r="AO7" s="24"/>
+      <c r="AP7" s="24"/>
+      <c r="AQ7" s="24"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="39">
-      <c r="A8" s="28" t="s">
+      <c r="A8" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="B8" s="29"/>
-      <c r="C8" s="29"/>
-      <c r="D8" s="29"/>
-      <c r="E8" s="29"/>
-      <c r="F8" s="29"/>
-      <c r="G8" s="29"/>
-      <c r="H8" s="30"/>
+      <c r="B8" s="30"/>
+      <c r="C8" s="30"/>
+      <c r="D8" s="30"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="30"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="31"/>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
-      <c r="L8" s="2"/>
-      <c r="M8" s="2"/>
+      <c r="K8" s="3"/>
+      <c r="L8" s="3"/>
+      <c r="M8" s="3"/>
       <c r="N8" s="2"/>
       <c r="O8" s="2"/>
       <c r="P8" s="2"/>
@@ -1565,23 +1571,23 @@
       <c r="AQ8" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="24">
-      <c r="A9" s="31" t="s">
+      <c r="A9" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="32"/>
-      <c r="C9" s="33"/>
-      <c r="D9" s="34" t="s">
+      <c r="B9" s="33"/>
+      <c r="C9" s="34"/>
+      <c r="D9" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="E9" s="34"/>
-      <c r="F9" s="34"/>
-      <c r="G9" s="34"/>
-      <c r="H9" s="35"/>
+      <c r="E9" s="35"/>
+      <c r="F9" s="35"/>
+      <c r="G9" s="35"/>
+      <c r="H9" s="36"/>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
-      <c r="L9" s="2"/>
-      <c r="M9" s="2"/>
+      <c r="K9" s="3"/>
+      <c r="L9" s="3"/>
+      <c r="M9" s="3"/>
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
       <c r="P9" s="2"/>
@@ -1614,23 +1620,23 @@
       <c r="AQ9" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
-      <c r="A10" s="31" t="s">
+      <c r="A10" s="32" t="s">
         <v>27</v>
       </c>
-      <c r="B10" s="32"/>
-      <c r="C10" s="34"/>
-      <c r="D10" s="34"/>
-      <c r="E10" s="34" t="s">
+      <c r="B10" s="33"/>
+      <c r="C10" s="35"/>
+      <c r="D10" s="35"/>
+      <c r="E10" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="F10" s="34"/>
-      <c r="G10" s="34"/>
-      <c r="H10" s="35"/>
+      <c r="F10" s="35"/>
+      <c r="G10" s="35"/>
+      <c r="H10" s="36"/>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
-      <c r="K10" s="2"/>
-      <c r="L10" s="2"/>
-      <c r="M10" s="2"/>
+      <c r="K10" s="3"/>
+      <c r="L10" s="3"/>
+      <c r="M10" s="3"/>
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
       <c r="P10" s="2"/>
@@ -1663,25 +1669,25 @@
       <c r="AQ10" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
-      <c r="A11" s="31" t="s">
+      <c r="A11" s="32" t="s">
         <v>28</v>
       </c>
-      <c r="B11" s="32"/>
-      <c r="C11" s="34"/>
-      <c r="D11" s="34"/>
-      <c r="E11" s="34" t="s">
+      <c r="B11" s="33"/>
+      <c r="C11" s="35"/>
+      <c r="D11" s="35"/>
+      <c r="E11" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="F11" s="34" t="s">
+      <c r="F11" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="G11" s="34"/>
-      <c r="H11" s="35"/>
+      <c r="G11" s="35"/>
+      <c r="H11" s="36"/>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
-      <c r="K11" s="2"/>
-      <c r="L11" s="2"/>
-      <c r="M11" s="2"/>
+      <c r="K11" s="3"/>
+      <c r="L11" s="3"/>
+      <c r="M11" s="3"/>
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
       <c r="P11" s="2"/>
@@ -1714,23 +1720,23 @@
       <c r="AQ11" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
-      <c r="A12" s="31" t="s">
+      <c r="A12" s="32" t="s">
         <v>29</v>
       </c>
-      <c r="B12" s="32"/>
-      <c r="C12" s="34"/>
-      <c r="D12" s="34"/>
-      <c r="E12" s="34"/>
-      <c r="F12" s="34"/>
-      <c r="G12" s="34" t="s">
+      <c r="B12" s="33"/>
+      <c r="C12" s="35"/>
+      <c r="D12" s="35"/>
+      <c r="E12" s="35"/>
+      <c r="F12" s="35"/>
+      <c r="G12" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="H12" s="35"/>
+      <c r="H12" s="36"/>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
-      <c r="K12" s="2"/>
-      <c r="L12" s="2"/>
-      <c r="M12" s="2"/>
+      <c r="K12" s="3"/>
+      <c r="L12" s="3"/>
+      <c r="M12" s="3"/>
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
       <c r="P12" s="2"/>
@@ -1763,23 +1769,23 @@
       <c r="AQ12" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
-      <c r="A13" s="31" t="s">
+      <c r="A13" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="B13" s="32"/>
-      <c r="C13" s="34"/>
-      <c r="D13" s="34"/>
-      <c r="E13" s="34"/>
-      <c r="F13" s="34"/>
-      <c r="G13" s="34"/>
-      <c r="H13" s="35" t="s">
+      <c r="B13" s="33"/>
+      <c r="C13" s="35"/>
+      <c r="D13" s="35"/>
+      <c r="E13" s="35"/>
+      <c r="F13" s="35"/>
+      <c r="G13" s="35"/>
+      <c r="H13" s="36" t="s">
         <v>26</v>
       </c>
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
-      <c r="K13" s="2"/>
-      <c r="L13" s="2"/>
-      <c r="M13" s="2"/>
+      <c r="K13" s="3"/>
+      <c r="L13" s="3"/>
+      <c r="M13" s="3"/>
       <c r="N13" s="2"/>
       <c r="O13" s="2"/>
       <c r="P13" s="2"/>
@@ -1812,23 +1818,23 @@
       <c r="AQ13" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
-      <c r="A14" s="31" t="s">
+      <c r="A14" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="B14" s="32"/>
-      <c r="C14" s="34"/>
-      <c r="D14" s="34"/>
-      <c r="E14" s="34"/>
-      <c r="F14" s="34"/>
-      <c r="G14" s="34"/>
-      <c r="H14" s="35" t="s">
+      <c r="B14" s="33"/>
+      <c r="C14" s="35"/>
+      <c r="D14" s="35"/>
+      <c r="E14" s="35"/>
+      <c r="F14" s="35"/>
+      <c r="G14" s="35"/>
+      <c r="H14" s="36" t="s">
         <v>26</v>
       </c>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
-      <c r="K14" s="2"/>
-      <c r="L14" s="2"/>
-      <c r="M14" s="2"/>
+      <c r="K14" s="3"/>
+      <c r="L14" s="3"/>
+      <c r="M14" s="3"/>
       <c r="N14" s="2"/>
       <c r="O14" s="2"/>
       <c r="P14" s="2"/>
@@ -1861,25 +1867,25 @@
       <c r="AQ14" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
-      <c r="A15" s="31" t="s">
+      <c r="A15" s="32" t="s">
         <v>32</v>
       </c>
-      <c r="B15" s="32"/>
-      <c r="C15" s="34" t="s">
+      <c r="B15" s="33"/>
+      <c r="C15" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="D15" s="34"/>
-      <c r="E15" s="34"/>
-      <c r="F15" s="34" t="s">
+      <c r="D15" s="35"/>
+      <c r="E15" s="35"/>
+      <c r="F15" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="G15" s="34"/>
-      <c r="H15" s="35"/>
+      <c r="G15" s="35"/>
+      <c r="H15" s="36"/>
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
-      <c r="K15" s="2"/>
-      <c r="L15" s="2"/>
-      <c r="M15" s="2"/>
+      <c r="K15" s="3"/>
+      <c r="L15" s="3"/>
+      <c r="M15" s="3"/>
       <c r="N15" s="2"/>
       <c r="O15" s="2"/>
       <c r="P15" s="2"/>
@@ -1912,25 +1918,25 @@
       <c r="AQ15" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
-      <c r="A16" s="31" t="s">
+      <c r="A16" s="32" t="s">
         <v>33</v>
       </c>
-      <c r="B16" s="32"/>
-      <c r="C16" s="34"/>
-      <c r="D16" s="34"/>
-      <c r="E16" s="34" t="s">
+      <c r="B16" s="33"/>
+      <c r="C16" s="35"/>
+      <c r="D16" s="35"/>
+      <c r="E16" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="F16" s="34" t="s">
+      <c r="F16" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="G16" s="34"/>
-      <c r="H16" s="35"/>
+      <c r="G16" s="35"/>
+      <c r="H16" s="36"/>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
-      <c r="K16" s="2"/>
-      <c r="L16" s="2"/>
-      <c r="M16" s="2"/>
+      <c r="K16" s="3"/>
+      <c r="L16" s="3"/>
+      <c r="M16" s="3"/>
       <c r="N16" s="2"/>
       <c r="O16" s="2"/>
       <c r="P16" s="2"/>
@@ -1963,23 +1969,23 @@
       <c r="AQ16" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
-      <c r="A17" s="31" t="s">
+      <c r="A17" s="32" t="s">
         <v>34</v>
       </c>
-      <c r="B17" s="32"/>
-      <c r="C17" s="34" t="s">
+      <c r="B17" s="33"/>
+      <c r="C17" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="D17" s="34"/>
-      <c r="E17" s="34"/>
-      <c r="F17" s="34"/>
-      <c r="G17" s="34"/>
-      <c r="H17" s="35"/>
+      <c r="D17" s="35"/>
+      <c r="E17" s="35"/>
+      <c r="F17" s="35"/>
+      <c r="G17" s="35"/>
+      <c r="H17" s="36"/>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
-      <c r="K17" s="2"/>
-      <c r="L17" s="2"/>
-      <c r="M17" s="2"/>
+      <c r="K17" s="3"/>
+      <c r="L17" s="3"/>
+      <c r="M17" s="3"/>
       <c r="N17" s="2"/>
       <c r="O17" s="2"/>
       <c r="P17" s="2"/>
@@ -2012,23 +2018,23 @@
       <c r="AQ17" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
-      <c r="A18" s="31" t="s">
+      <c r="A18" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="B18" s="32"/>
-      <c r="C18" s="34"/>
-      <c r="D18" s="34"/>
-      <c r="E18" s="34"/>
-      <c r="F18" s="34"/>
-      <c r="G18" s="34"/>
-      <c r="H18" s="35" t="s">
+      <c r="B18" s="33"/>
+      <c r="C18" s="35"/>
+      <c r="D18" s="35"/>
+      <c r="E18" s="35"/>
+      <c r="F18" s="35"/>
+      <c r="G18" s="35"/>
+      <c r="H18" s="36" t="s">
         <v>26</v>
       </c>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
-      <c r="K18" s="2"/>
-      <c r="L18" s="2"/>
-      <c r="M18" s="2"/>
+      <c r="K18" s="3"/>
+      <c r="L18" s="3"/>
+      <c r="M18" s="3"/>
       <c r="N18" s="2"/>
       <c r="O18" s="2"/>
       <c r="P18" s="2"/>
@@ -2061,23 +2067,23 @@
       <c r="AQ18" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
-      <c r="A19" s="31" t="s">
+      <c r="A19" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="B19" s="32"/>
-      <c r="C19" s="34"/>
-      <c r="D19" s="34"/>
-      <c r="E19" s="34"/>
-      <c r="F19" s="34"/>
-      <c r="G19" s="34"/>
-      <c r="H19" s="35" t="s">
+      <c r="B19" s="33"/>
+      <c r="C19" s="35"/>
+      <c r="D19" s="35"/>
+      <c r="E19" s="35"/>
+      <c r="F19" s="35"/>
+      <c r="G19" s="35"/>
+      <c r="H19" s="36" t="s">
         <v>26</v>
       </c>
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
-      <c r="K19" s="2"/>
-      <c r="L19" s="2"/>
-      <c r="M19" s="2"/>
+      <c r="K19" s="3"/>
+      <c r="L19" s="3"/>
+      <c r="M19" s="3"/>
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
       <c r="P19" s="2"/>
@@ -2110,23 +2116,23 @@
       <c r="AQ19" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
-      <c r="A20" s="31" t="s">
+      <c r="A20" s="32" t="s">
         <v>37</v>
       </c>
-      <c r="B20" s="32"/>
-      <c r="C20" s="34"/>
-      <c r="D20" s="34"/>
-      <c r="E20" s="34"/>
-      <c r="F20" s="34"/>
-      <c r="G20" s="34"/>
-      <c r="H20" s="35" t="s">
+      <c r="B20" s="33"/>
+      <c r="C20" s="35"/>
+      <c r="D20" s="35"/>
+      <c r="E20" s="35"/>
+      <c r="F20" s="35"/>
+      <c r="G20" s="35"/>
+      <c r="H20" s="36" t="s">
         <v>26</v>
       </c>
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
-      <c r="K20" s="2"/>
-      <c r="L20" s="2"/>
-      <c r="M20" s="2"/>
+      <c r="K20" s="3"/>
+      <c r="L20" s="3"/>
+      <c r="M20" s="3"/>
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
       <c r="P20" s="2"/>
@@ -2159,25 +2165,25 @@
       <c r="AQ20" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
-      <c r="A21" s="31" t="s">
+      <c r="A21" s="32" t="s">
         <v>38</v>
       </c>
-      <c r="B21" s="32"/>
-      <c r="C21" s="34"/>
-      <c r="D21" s="34"/>
-      <c r="E21" s="34"/>
-      <c r="F21" s="34"/>
-      <c r="G21" s="35" t="s">
+      <c r="B21" s="33"/>
+      <c r="C21" s="35"/>
+      <c r="D21" s="35"/>
+      <c r="E21" s="35"/>
+      <c r="F21" s="35"/>
+      <c r="G21" s="36" t="s">
         <v>26</v>
       </c>
-      <c r="H21" s="35" t="s">
+      <c r="H21" s="36" t="s">
         <v>26</v>
       </c>
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
-      <c r="K21" s="2"/>
-      <c r="L21" s="2"/>
-      <c r="M21" s="2"/>
+      <c r="K21" s="3"/>
+      <c r="L21" s="3"/>
+      <c r="M21" s="3"/>
       <c r="N21" s="2"/>
       <c r="O21" s="2"/>
       <c r="P21" s="2"/>
@@ -2210,21 +2216,21 @@
       <c r="AQ21" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="22.5">
-      <c r="A22" s="36" t="s">
+      <c r="A22" s="37" t="s">
         <v>39</v>
       </c>
-      <c r="B22" s="37"/>
-      <c r="C22" s="37"/>
-      <c r="D22" s="37"/>
-      <c r="E22" s="37"/>
-      <c r="F22" s="37"/>
-      <c r="G22" s="37"/>
-      <c r="H22" s="38"/>
+      <c r="B22" s="38"/>
+      <c r="C22" s="38"/>
+      <c r="D22" s="38"/>
+      <c r="E22" s="38"/>
+      <c r="F22" s="38"/>
+      <c r="G22" s="38"/>
+      <c r="H22" s="39"/>
       <c r="I22" s="2"/>
       <c r="J22" s="2"/>
-      <c r="K22" s="2"/>
-      <c r="L22" s="2"/>
-      <c r="M22" s="2"/>
+      <c r="K22" s="3"/>
+      <c r="L22" s="3"/>
+      <c r="M22" s="3"/>
       <c r="N22" s="2"/>
       <c r="O22" s="2"/>
       <c r="P22" s="2"/>
@@ -2257,29 +2263,29 @@
       <c r="AQ22" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
-      <c r="A23" s="31" t="s">
+      <c r="A23" s="32" t="s">
         <v>40</v>
       </c>
-      <c r="B23" s="32"/>
-      <c r="C23" s="34" t="s">
+      <c r="B23" s="33"/>
+      <c r="C23" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="D23" s="34" t="s">
+      <c r="D23" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="E23" s="34" t="s">
+      <c r="E23" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="F23" s="34" t="s">
+      <c r="F23" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="G23" s="34"/>
-      <c r="H23" s="35"/>
+      <c r="G23" s="35"/>
+      <c r="H23" s="36"/>
       <c r="I23" s="2"/>
       <c r="J23" s="2"/>
-      <c r="K23" s="2"/>
-      <c r="L23" s="2"/>
-      <c r="M23" s="2"/>
+      <c r="K23" s="3"/>
+      <c r="L23" s="3"/>
+      <c r="M23" s="3"/>
       <c r="N23" s="2"/>
       <c r="O23" s="2"/>
       <c r="P23" s="2"/>
@@ -2312,21 +2318,21 @@
       <c r="AQ23" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
-      <c r="A24" s="31" t="s">
+      <c r="A24" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="B24" s="32"/>
-      <c r="C24" s="34"/>
-      <c r="D24" s="34"/>
-      <c r="E24" s="34"/>
-      <c r="F24" s="34"/>
-      <c r="G24" s="34"/>
-      <c r="H24" s="35"/>
+      <c r="B24" s="33"/>
+      <c r="C24" s="35"/>
+      <c r="D24" s="35"/>
+      <c r="E24" s="35"/>
+      <c r="F24" s="35"/>
+      <c r="G24" s="35"/>
+      <c r="H24" s="36"/>
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
-      <c r="K24" s="2"/>
-      <c r="L24" s="2"/>
-      <c r="M24" s="2"/>
+      <c r="K24" s="3"/>
+      <c r="L24" s="3"/>
+      <c r="M24" s="3"/>
       <c r="N24" s="2"/>
       <c r="O24" s="2"/>
       <c r="P24" s="2"/>
@@ -2359,19 +2365,19 @@
       <c r="AQ24" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="39.95">
-      <c r="A25" s="31"/>
-      <c r="B25" s="32"/>
-      <c r="C25" s="34"/>
-      <c r="D25" s="34"/>
-      <c r="E25" s="34"/>
-      <c r="F25" s="34"/>
-      <c r="G25" s="34"/>
-      <c r="H25" s="35"/>
+      <c r="A25" s="32"/>
+      <c r="B25" s="33"/>
+      <c r="C25" s="35"/>
+      <c r="D25" s="35"/>
+      <c r="E25" s="35"/>
+      <c r="F25" s="35"/>
+      <c r="G25" s="35"/>
+      <c r="H25" s="36"/>
       <c r="I25" s="2"/>
       <c r="J25" s="2"/>
-      <c r="K25" s="2"/>
-      <c r="L25" s="2"/>
-      <c r="M25" s="2"/>
+      <c r="K25" s="3"/>
+      <c r="L25" s="3"/>
+      <c r="M25" s="3"/>
       <c r="N25" s="2"/>
       <c r="O25" s="2"/>
       <c r="P25" s="2"/>
@@ -2404,21 +2410,21 @@
       <c r="AQ25" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
-      <c r="A26" s="36" t="s">
+      <c r="A26" s="37" t="s">
         <v>42</v>
       </c>
-      <c r="B26" s="37"/>
-      <c r="C26" s="37"/>
-      <c r="D26" s="37"/>
-      <c r="E26" s="37"/>
-      <c r="F26" s="37"/>
-      <c r="G26" s="37"/>
-      <c r="H26" s="38"/>
+      <c r="B26" s="38"/>
+      <c r="C26" s="38"/>
+      <c r="D26" s="38"/>
+      <c r="E26" s="38"/>
+      <c r="F26" s="38"/>
+      <c r="G26" s="38"/>
+      <c r="H26" s="39"/>
       <c r="I26" s="2"/>
       <c r="J26" s="2"/>
-      <c r="K26" s="2"/>
-      <c r="L26" s="2"/>
-      <c r="M26" s="2"/>
+      <c r="K26" s="3"/>
+      <c r="L26" s="3"/>
+      <c r="M26" s="3"/>
       <c r="N26" s="2"/>
       <c r="O26" s="2"/>
       <c r="P26" s="2"/>
@@ -2451,31 +2457,29 @@
       <c r="AQ26" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="39.95">
-      <c r="A27" s="31" t="s">
+      <c r="A27" s="32" t="s">
         <v>43</v>
       </c>
-      <c r="B27" s="32"/>
-      <c r="C27" s="39" t="s">
-        <v>44</v>
-      </c>
-      <c r="D27" s="34" t="s">
+      <c r="B27" s="33"/>
+      <c r="C27" s="35"/>
+      <c r="D27" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="E27" s="34" t="s">
+      <c r="E27" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="F27" s="34" t="s">
+      <c r="F27" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="G27" s="34"/>
-      <c r="H27" s="35" t="s">
+      <c r="G27" s="35"/>
+      <c r="H27" s="36" t="s">
         <v>26</v>
       </c>
       <c r="I27" s="2"/>
       <c r="J27" s="2"/>
-      <c r="K27" s="2"/>
-      <c r="L27" s="2"/>
-      <c r="M27" s="2"/>
+      <c r="K27" s="3"/>
+      <c r="L27" s="3"/>
+      <c r="M27" s="3"/>
       <c r="N27" s="2"/>
       <c r="O27" s="2"/>
       <c r="P27" s="2"/>
@@ -2508,25 +2512,25 @@
       <c r="AQ27" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="39.95">
-      <c r="A28" s="31" t="s">
-        <v>45</v>
-      </c>
-      <c r="B28" s="32"/>
-      <c r="C28" s="34"/>
-      <c r="D28" s="34"/>
-      <c r="E28" s="34" t="s">
+      <c r="A28" s="32" t="s">
+        <v>44</v>
+      </c>
+      <c r="B28" s="33"/>
+      <c r="C28" s="35"/>
+      <c r="D28" s="35"/>
+      <c r="E28" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="F28" s="34" t="s">
+      <c r="F28" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="G28" s="34"/>
-      <c r="H28" s="35"/>
+      <c r="G28" s="35"/>
+      <c r="H28" s="36"/>
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
-      <c r="K28" s="2"/>
-      <c r="L28" s="2"/>
-      <c r="M28" s="2"/>
+      <c r="K28" s="3"/>
+      <c r="L28" s="3"/>
+      <c r="M28" s="3"/>
       <c r="N28" s="2"/>
       <c r="O28" s="2"/>
       <c r="P28" s="2"/>
@@ -2559,23 +2563,23 @@
       <c r="AQ28" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="39.95">
-      <c r="A29" s="31" t="s">
-        <v>46</v>
-      </c>
-      <c r="B29" s="32"/>
-      <c r="C29" s="34"/>
-      <c r="D29" s="34"/>
-      <c r="E29" s="34"/>
-      <c r="F29" s="34" t="s">
+      <c r="A29" s="32" t="s">
+        <v>45</v>
+      </c>
+      <c r="B29" s="33"/>
+      <c r="C29" s="35"/>
+      <c r="D29" s="35"/>
+      <c r="E29" s="35"/>
+      <c r="F29" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="G29" s="34"/>
-      <c r="H29" s="35"/>
+      <c r="G29" s="35"/>
+      <c r="H29" s="36"/>
       <c r="I29" s="2"/>
       <c r="J29" s="2"/>
-      <c r="K29" s="2"/>
-      <c r="L29" s="2"/>
-      <c r="M29" s="2"/>
+      <c r="K29" s="3"/>
+      <c r="L29" s="3"/>
+      <c r="M29" s="3"/>
       <c r="N29" s="2"/>
       <c r="O29" s="2"/>
       <c r="P29" s="2"/>
@@ -2618,9 +2622,9 @@
       <c r="H30" s="43"/>
       <c r="I30" s="2"/>
       <c r="J30" s="2"/>
-      <c r="K30" s="2"/>
-      <c r="L30" s="2"/>
-      <c r="M30" s="2"/>
+      <c r="K30" s="3"/>
+      <c r="L30" s="3"/>
+      <c r="M30" s="3"/>
       <c r="N30" s="2"/>
       <c r="O30" s="2"/>
       <c r="P30" s="2"/>
@@ -2663,9 +2667,9 @@
       <c r="H31" s="46"/>
       <c r="I31" s="2"/>
       <c r="J31" s="2"/>
-      <c r="K31" s="2"/>
-      <c r="L31" s="2"/>
-      <c r="M31" s="2"/>
+      <c r="K31" s="3"/>
+      <c r="L31" s="3"/>
+      <c r="M31" s="3"/>
       <c r="N31" s="2"/>
       <c r="O31" s="2"/>
       <c r="P31" s="2"/>
@@ -2698,19 +2702,19 @@
       <c r="AQ31" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
-      <c r="A32" s="2"/>
-      <c r="B32" s="2"/>
-      <c r="C32" s="2"/>
-      <c r="D32" s="2"/>
-      <c r="E32" s="2"/>
-      <c r="F32" s="2"/>
-      <c r="G32" s="2"/>
-      <c r="H32" s="2"/>
+      <c r="A32" s="3"/>
+      <c r="B32" s="3"/>
+      <c r="C32" s="3"/>
+      <c r="D32" s="3"/>
+      <c r="E32" s="3"/>
+      <c r="F32" s="3"/>
+      <c r="G32" s="3"/>
+      <c r="H32" s="3"/>
       <c r="I32" s="2"/>
       <c r="J32" s="2"/>
-      <c r="K32" s="2"/>
-      <c r="L32" s="2"/>
-      <c r="M32" s="2"/>
+      <c r="K32" s="3"/>
+      <c r="L32" s="3"/>
+      <c r="M32" s="3"/>
       <c r="N32" s="2"/>
       <c r="O32" s="2"/>
       <c r="P32" s="2"/>
@@ -2743,19 +2747,19 @@
       <c r="AQ32" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75">
-      <c r="A33" s="2"/>
-      <c r="B33" s="2"/>
-      <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
-      <c r="E33" s="2"/>
-      <c r="F33" s="2"/>
-      <c r="G33" s="2"/>
-      <c r="H33" s="2"/>
+      <c r="A33" s="3"/>
+      <c r="B33" s="3"/>
+      <c r="C33" s="3"/>
+      <c r="D33" s="3"/>
+      <c r="E33" s="3"/>
+      <c r="F33" s="3"/>
+      <c r="G33" s="3"/>
+      <c r="H33" s="3"/>
       <c r="I33" s="2"/>
       <c r="J33" s="2"/>
-      <c r="K33" s="2"/>
-      <c r="L33" s="2"/>
-      <c r="M33" s="2"/>
+      <c r="K33" s="3"/>
+      <c r="L33" s="3"/>
+      <c r="M33" s="3"/>
       <c r="N33" s="2"/>
       <c r="O33" s="2"/>
       <c r="P33" s="2"/>
@@ -2788,19 +2792,19 @@
       <c r="AQ33" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
-      <c r="A34" s="2"/>
-      <c r="B34" s="2"/>
-      <c r="C34" s="2"/>
-      <c r="D34" s="2"/>
-      <c r="E34" s="2"/>
-      <c r="F34" s="2"/>
-      <c r="G34" s="2"/>
-      <c r="H34" s="2"/>
+      <c r="A34" s="3"/>
+      <c r="B34" s="3"/>
+      <c r="C34" s="3"/>
+      <c r="D34" s="3"/>
+      <c r="E34" s="3"/>
+      <c r="F34" s="3"/>
+      <c r="G34" s="3"/>
+      <c r="H34" s="3"/>
       <c r="I34" s="2"/>
       <c r="J34" s="2"/>
-      <c r="K34" s="2"/>
-      <c r="L34" s="2"/>
-      <c r="M34" s="2"/>
+      <c r="K34" s="3"/>
+      <c r="L34" s="3"/>
+      <c r="M34" s="3"/>
       <c r="N34" s="2"/>
       <c r="O34" s="2"/>
       <c r="P34" s="2"/>
@@ -2833,19 +2837,19 @@
       <c r="AQ34" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75">
-      <c r="A35" s="2"/>
-      <c r="B35" s="2"/>
-      <c r="C35" s="2"/>
-      <c r="D35" s="2"/>
-      <c r="E35" s="2"/>
-      <c r="F35" s="2"/>
-      <c r="G35" s="2"/>
-      <c r="H35" s="2"/>
+      <c r="A35" s="3"/>
+      <c r="B35" s="3"/>
+      <c r="C35" s="3"/>
+      <c r="D35" s="3"/>
+      <c r="E35" s="3"/>
+      <c r="F35" s="3"/>
+      <c r="G35" s="3"/>
+      <c r="H35" s="3"/>
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
-      <c r="K35" s="2"/>
-      <c r="L35" s="2"/>
-      <c r="M35" s="2"/>
+      <c r="K35" s="3"/>
+      <c r="L35" s="3"/>
+      <c r="M35" s="3"/>
       <c r="N35" s="2"/>
       <c r="O35" s="2"/>
       <c r="P35" s="2"/>
@@ -2878,19 +2882,19 @@
       <c r="AQ35" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75">
-      <c r="A36" s="2"/>
-      <c r="B36" s="2"/>
-      <c r="C36" s="2"/>
-      <c r="D36" s="2"/>
-      <c r="E36" s="2"/>
-      <c r="F36" s="2"/>
-      <c r="G36" s="2"/>
-      <c r="H36" s="2"/>
+      <c r="A36" s="3"/>
+      <c r="B36" s="3"/>
+      <c r="C36" s="3"/>
+      <c r="D36" s="3"/>
+      <c r="E36" s="3"/>
+      <c r="F36" s="3"/>
+      <c r="G36" s="3"/>
+      <c r="H36" s="3"/>
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
-      <c r="K36" s="2"/>
-      <c r="L36" s="2"/>
-      <c r="M36" s="2"/>
+      <c r="K36" s="3"/>
+      <c r="L36" s="3"/>
+      <c r="M36" s="3"/>
       <c r="N36" s="2"/>
       <c r="O36" s="2"/>
       <c r="P36" s="2"/>
@@ -2923,19 +2927,19 @@
       <c r="AQ36" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75">
-      <c r="A37" s="2"/>
-      <c r="B37" s="2"/>
-      <c r="C37" s="2"/>
-      <c r="D37" s="2"/>
-      <c r="E37" s="2"/>
-      <c r="F37" s="2"/>
-      <c r="G37" s="2"/>
-      <c r="H37" s="2"/>
+      <c r="A37" s="3"/>
+      <c r="B37" s="3"/>
+      <c r="C37" s="3"/>
+      <c r="D37" s="3"/>
+      <c r="E37" s="3"/>
+      <c r="F37" s="3"/>
+      <c r="G37" s="3"/>
+      <c r="H37" s="3"/>
       <c r="I37" s="2"/>
       <c r="J37" s="2"/>
-      <c r="K37" s="2"/>
-      <c r="L37" s="2"/>
-      <c r="M37" s="2"/>
+      <c r="K37" s="3"/>
+      <c r="L37" s="3"/>
+      <c r="M37" s="3"/>
       <c r="N37" s="2"/>
       <c r="O37" s="2"/>
       <c r="P37" s="2"/>
@@ -2968,19 +2972,19 @@
       <c r="AQ37" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18.75">
-      <c r="A38" s="2"/>
-      <c r="B38" s="2"/>
-      <c r="C38" s="2"/>
-      <c r="D38" s="2"/>
-      <c r="E38" s="2"/>
-      <c r="F38" s="2"/>
-      <c r="G38" s="2"/>
-      <c r="H38" s="2"/>
+      <c r="A38" s="3"/>
+      <c r="B38" s="3"/>
+      <c r="C38" s="3"/>
+      <c r="D38" s="3"/>
+      <c r="E38" s="3"/>
+      <c r="F38" s="3"/>
+      <c r="G38" s="3"/>
+      <c r="H38" s="3"/>
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
-      <c r="K38" s="2"/>
-      <c r="L38" s="2"/>
-      <c r="M38" s="2"/>
+      <c r="K38" s="3"/>
+      <c r="L38" s="3"/>
+      <c r="M38" s="3"/>
       <c r="N38" s="2"/>
       <c r="O38" s="2"/>
       <c r="P38" s="2"/>
@@ -3013,19 +3017,19 @@
       <c r="AQ38" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18.75">
-      <c r="A39" s="2"/>
-      <c r="B39" s="2"/>
-      <c r="C39" s="2"/>
-      <c r="D39" s="2"/>
-      <c r="E39" s="2"/>
-      <c r="F39" s="2"/>
-      <c r="G39" s="2"/>
-      <c r="H39" s="2"/>
+      <c r="A39" s="3"/>
+      <c r="B39" s="3"/>
+      <c r="C39" s="3"/>
+      <c r="D39" s="3"/>
+      <c r="E39" s="3"/>
+      <c r="F39" s="3"/>
+      <c r="G39" s="3"/>
+      <c r="H39" s="3"/>
       <c r="I39" s="2"/>
       <c r="J39" s="2"/>
-      <c r="K39" s="2"/>
-      <c r="L39" s="2"/>
-      <c r="M39" s="2"/>
+      <c r="K39" s="3"/>
+      <c r="L39" s="3"/>
+      <c r="M39" s="3"/>
       <c r="N39" s="2"/>
       <c r="O39" s="2"/>
       <c r="P39" s="2"/>
@@ -3058,19 +3062,19 @@
       <c r="AQ39" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18.75">
-      <c r="A40" s="2"/>
-      <c r="B40" s="2"/>
-      <c r="C40" s="2"/>
-      <c r="D40" s="2"/>
-      <c r="E40" s="2"/>
-      <c r="F40" s="2"/>
-      <c r="G40" s="2"/>
-      <c r="H40" s="2"/>
+      <c r="A40" s="3"/>
+      <c r="B40" s="3"/>
+      <c r="C40" s="3"/>
+      <c r="D40" s="3"/>
+      <c r="E40" s="3"/>
+      <c r="F40" s="3"/>
+      <c r="G40" s="3"/>
+      <c r="H40" s="3"/>
       <c r="I40" s="2"/>
       <c r="J40" s="2"/>
-      <c r="K40" s="2"/>
-      <c r="L40" s="2"/>
-      <c r="M40" s="2"/>
+      <c r="K40" s="3"/>
+      <c r="L40" s="3"/>
+      <c r="M40" s="3"/>
       <c r="N40" s="2"/>
       <c r="O40" s="2"/>
       <c r="P40" s="2"/>
@@ -3103,19 +3107,19 @@
       <c r="AQ40" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18.75">
-      <c r="A41" s="2"/>
-      <c r="B41" s="2"/>
-      <c r="C41" s="2"/>
-      <c r="D41" s="2"/>
-      <c r="E41" s="2"/>
-      <c r="F41" s="2"/>
-      <c r="G41" s="2"/>
-      <c r="H41" s="2"/>
+      <c r="A41" s="3"/>
+      <c r="B41" s="3"/>
+      <c r="C41" s="3"/>
+      <c r="D41" s="3"/>
+      <c r="E41" s="3"/>
+      <c r="F41" s="3"/>
+      <c r="G41" s="3"/>
+      <c r="H41" s="3"/>
       <c r="I41" s="2"/>
       <c r="J41" s="2"/>
-      <c r="K41" s="2"/>
-      <c r="L41" s="2"/>
-      <c r="M41" s="2"/>
+      <c r="K41" s="3"/>
+      <c r="L41" s="3"/>
+      <c r="M41" s="3"/>
       <c r="N41" s="2"/>
       <c r="O41" s="2"/>
       <c r="P41" s="2"/>
@@ -3148,19 +3152,19 @@
       <c r="AQ41" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18.75">
-      <c r="A42" s="2"/>
-      <c r="B42" s="2"/>
-      <c r="C42" s="2"/>
-      <c r="D42" s="2"/>
-      <c r="E42" s="2"/>
-      <c r="F42" s="2"/>
-      <c r="G42" s="2"/>
-      <c r="H42" s="2"/>
+      <c r="A42" s="3"/>
+      <c r="B42" s="3"/>
+      <c r="C42" s="3"/>
+      <c r="D42" s="3"/>
+      <c r="E42" s="3"/>
+      <c r="F42" s="3"/>
+      <c r="G42" s="3"/>
+      <c r="H42" s="3"/>
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
-      <c r="K42" s="2"/>
-      <c r="L42" s="2"/>
-      <c r="M42" s="2"/>
+      <c r="K42" s="3"/>
+      <c r="L42" s="3"/>
+      <c r="M42" s="3"/>
       <c r="N42" s="2"/>
       <c r="O42" s="2"/>
       <c r="P42" s="2"/>
@@ -3193,19 +3197,19 @@
       <c r="AQ42" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="18.75">
-      <c r="A43" s="2"/>
-      <c r="B43" s="2"/>
-      <c r="C43" s="2"/>
-      <c r="D43" s="2"/>
-      <c r="E43" s="2"/>
-      <c r="F43" s="2"/>
-      <c r="G43" s="2"/>
-      <c r="H43" s="2"/>
+      <c r="A43" s="3"/>
+      <c r="B43" s="3"/>
+      <c r="C43" s="3"/>
+      <c r="D43" s="3"/>
+      <c r="E43" s="3"/>
+      <c r="F43" s="3"/>
+      <c r="G43" s="3"/>
+      <c r="H43" s="3"/>
       <c r="I43" s="2"/>
       <c r="J43" s="2"/>
-      <c r="K43" s="2"/>
-      <c r="L43" s="2"/>
-      <c r="M43" s="2"/>
+      <c r="K43" s="3"/>
+      <c r="L43" s="3"/>
+      <c r="M43" s="3"/>
       <c r="N43" s="2"/>
       <c r="O43" s="2"/>
       <c r="P43" s="2"/>
@@ -3238,19 +3242,19 @@
       <c r="AQ43" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="18.75">
-      <c r="A44" s="2"/>
-      <c r="B44" s="2"/>
-      <c r="C44" s="2"/>
-      <c r="D44" s="2"/>
-      <c r="E44" s="2"/>
-      <c r="F44" s="2"/>
-      <c r="G44" s="2"/>
-      <c r="H44" s="2"/>
+      <c r="A44" s="3"/>
+      <c r="B44" s="3"/>
+      <c r="C44" s="3"/>
+      <c r="D44" s="3"/>
+      <c r="E44" s="3"/>
+      <c r="F44" s="3"/>
+      <c r="G44" s="3"/>
+      <c r="H44" s="3"/>
       <c r="I44" s="2"/>
       <c r="J44" s="2"/>
-      <c r="K44" s="2"/>
-      <c r="L44" s="2"/>
-      <c r="M44" s="2"/>
+      <c r="K44" s="3"/>
+      <c r="L44" s="3"/>
+      <c r="M44" s="3"/>
       <c r="N44" s="2"/>
       <c r="O44" s="2"/>
       <c r="P44" s="2"/>
@@ -3283,19 +3287,19 @@
       <c r="AQ44" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="18.75">
-      <c r="A45" s="2"/>
-      <c r="B45" s="2"/>
-      <c r="C45" s="2"/>
-      <c r="D45" s="2"/>
-      <c r="E45" s="2"/>
-      <c r="F45" s="2"/>
-      <c r="G45" s="2"/>
-      <c r="H45" s="2"/>
+      <c r="A45" s="3"/>
+      <c r="B45" s="3"/>
+      <c r="C45" s="3"/>
+      <c r="D45" s="3"/>
+      <c r="E45" s="3"/>
+      <c r="F45" s="3"/>
+      <c r="G45" s="3"/>
+      <c r="H45" s="3"/>
       <c r="I45" s="2"/>
       <c r="J45" s="2"/>
-      <c r="K45" s="2"/>
-      <c r="L45" s="2"/>
-      <c r="M45" s="2"/>
+      <c r="K45" s="3"/>
+      <c r="L45" s="3"/>
+      <c r="M45" s="3"/>
       <c r="N45" s="2"/>
       <c r="O45" s="2"/>
       <c r="P45" s="2"/>
@@ -3328,19 +3332,19 @@
       <c r="AQ45" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="18.75">
-      <c r="A46" s="2"/>
-      <c r="B46" s="2"/>
-      <c r="C46" s="2"/>
-      <c r="D46" s="2"/>
-      <c r="E46" s="2"/>
-      <c r="F46" s="2"/>
-      <c r="G46" s="2"/>
-      <c r="H46" s="2"/>
+      <c r="A46" s="3"/>
+      <c r="B46" s="3"/>
+      <c r="C46" s="3"/>
+      <c r="D46" s="3"/>
+      <c r="E46" s="3"/>
+      <c r="F46" s="3"/>
+      <c r="G46" s="3"/>
+      <c r="H46" s="3"/>
       <c r="I46" s="2"/>
       <c r="J46" s="2"/>
-      <c r="K46" s="2"/>
-      <c r="L46" s="2"/>
-      <c r="M46" s="2"/>
+      <c r="K46" s="3"/>
+      <c r="L46" s="3"/>
+      <c r="M46" s="3"/>
       <c r="N46" s="2"/>
       <c r="O46" s="2"/>
       <c r="P46" s="2"/>
@@ -3373,19 +3377,19 @@
       <c r="AQ46" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="18.75">
-      <c r="A47" s="2"/>
-      <c r="B47" s="2"/>
-      <c r="C47" s="2"/>
-      <c r="D47" s="2"/>
-      <c r="E47" s="2"/>
-      <c r="F47" s="2"/>
-      <c r="G47" s="2"/>
-      <c r="H47" s="2"/>
+      <c r="A47" s="3"/>
+      <c r="B47" s="3"/>
+      <c r="C47" s="3"/>
+      <c r="D47" s="3"/>
+      <c r="E47" s="3"/>
+      <c r="F47" s="3"/>
+      <c r="G47" s="3"/>
+      <c r="H47" s="3"/>
       <c r="I47" s="2"/>
       <c r="J47" s="2"/>
-      <c r="K47" s="2"/>
-      <c r="L47" s="2"/>
-      <c r="M47" s="2"/>
+      <c r="K47" s="3"/>
+      <c r="L47" s="3"/>
+      <c r="M47" s="3"/>
       <c r="N47" s="2"/>
       <c r="O47" s="2"/>
       <c r="P47" s="2"/>
@@ -3418,19 +3422,19 @@
       <c r="AQ47" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="18.75">
-      <c r="A48" s="2"/>
-      <c r="B48" s="2"/>
-      <c r="C48" s="2"/>
-      <c r="D48" s="2"/>
-      <c r="E48" s="2"/>
-      <c r="F48" s="2"/>
-      <c r="G48" s="2"/>
-      <c r="H48" s="2"/>
+      <c r="A48" s="3"/>
+      <c r="B48" s="3"/>
+      <c r="C48" s="3"/>
+      <c r="D48" s="3"/>
+      <c r="E48" s="3"/>
+      <c r="F48" s="3"/>
+      <c r="G48" s="3"/>
+      <c r="H48" s="3"/>
       <c r="I48" s="2"/>
       <c r="J48" s="2"/>
-      <c r="K48" s="2"/>
-      <c r="L48" s="2"/>
-      <c r="M48" s="2"/>
+      <c r="K48" s="3"/>
+      <c r="L48" s="3"/>
+      <c r="M48" s="3"/>
       <c r="N48" s="2"/>
       <c r="O48" s="2"/>
       <c r="P48" s="2"/>
@@ -3463,19 +3467,19 @@
       <c r="AQ48" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="18.75">
-      <c r="A49" s="2"/>
-      <c r="B49" s="2"/>
-      <c r="C49" s="2"/>
-      <c r="D49" s="2"/>
-      <c r="E49" s="2"/>
-      <c r="F49" s="2"/>
-      <c r="G49" s="2"/>
-      <c r="H49" s="2"/>
+      <c r="A49" s="3"/>
+      <c r="B49" s="3"/>
+      <c r="C49" s="3"/>
+      <c r="D49" s="3"/>
+      <c r="E49" s="3"/>
+      <c r="F49" s="3"/>
+      <c r="G49" s="3"/>
+      <c r="H49" s="3"/>
       <c r="I49" s="2"/>
       <c r="J49" s="2"/>
-      <c r="K49" s="2"/>
-      <c r="L49" s="2"/>
-      <c r="M49" s="2"/>
+      <c r="K49" s="3"/>
+      <c r="L49" s="3"/>
+      <c r="M49" s="3"/>
       <c r="N49" s="2"/>
       <c r="O49" s="2"/>
       <c r="P49" s="2"/>
@@ -3508,19 +3512,19 @@
       <c r="AQ49" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="18.75">
-      <c r="A50" s="2"/>
-      <c r="B50" s="2"/>
-      <c r="C50" s="2"/>
-      <c r="D50" s="2"/>
-      <c r="E50" s="2"/>
-      <c r="F50" s="2"/>
-      <c r="G50" s="2"/>
-      <c r="H50" s="2"/>
+      <c r="A50" s="3"/>
+      <c r="B50" s="3"/>
+      <c r="C50" s="3"/>
+      <c r="D50" s="3"/>
+      <c r="E50" s="3"/>
+      <c r="F50" s="3"/>
+      <c r="G50" s="3"/>
+      <c r="H50" s="3"/>
       <c r="I50" s="2"/>
       <c r="J50" s="2"/>
-      <c r="K50" s="2"/>
-      <c r="L50" s="2"/>
-      <c r="M50" s="2"/>
+      <c r="K50" s="3"/>
+      <c r="L50" s="3"/>
+      <c r="M50" s="3"/>
       <c r="N50" s="2"/>
       <c r="O50" s="2"/>
       <c r="P50" s="2"/>
@@ -3553,19 +3557,19 @@
       <c r="AQ50" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="18.75">
-      <c r="A51" s="2"/>
-      <c r="B51" s="2"/>
-      <c r="C51" s="2"/>
-      <c r="D51" s="2"/>
-      <c r="E51" s="2"/>
-      <c r="F51" s="2"/>
-      <c r="G51" s="2"/>
-      <c r="H51" s="2"/>
+      <c r="A51" s="3"/>
+      <c r="B51" s="3"/>
+      <c r="C51" s="3"/>
+      <c r="D51" s="3"/>
+      <c r="E51" s="3"/>
+      <c r="F51" s="3"/>
+      <c r="G51" s="3"/>
+      <c r="H51" s="3"/>
       <c r="I51" s="2"/>
       <c r="J51" s="2"/>
-      <c r="K51" s="2"/>
-      <c r="L51" s="2"/>
-      <c r="M51" s="2"/>
+      <c r="K51" s="3"/>
+      <c r="L51" s="3"/>
+      <c r="M51" s="3"/>
       <c r="N51" s="2"/>
       <c r="O51" s="2"/>
       <c r="P51" s="2"/>
@@ -3598,19 +3602,19 @@
       <c r="AQ51" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="18.75">
-      <c r="A52" s="2"/>
-      <c r="B52" s="2"/>
-      <c r="C52" s="2"/>
-      <c r="D52" s="2"/>
-      <c r="E52" s="2"/>
-      <c r="F52" s="2"/>
-      <c r="G52" s="2"/>
-      <c r="H52" s="2"/>
+      <c r="A52" s="3"/>
+      <c r="B52" s="3"/>
+      <c r="C52" s="3"/>
+      <c r="D52" s="3"/>
+      <c r="E52" s="3"/>
+      <c r="F52" s="3"/>
+      <c r="G52" s="3"/>
+      <c r="H52" s="3"/>
       <c r="I52" s="2"/>
       <c r="J52" s="2"/>
-      <c r="K52" s="2"/>
-      <c r="L52" s="2"/>
-      <c r="M52" s="2"/>
+      <c r="K52" s="3"/>
+      <c r="L52" s="3"/>
+      <c r="M52" s="3"/>
       <c r="N52" s="2"/>
       <c r="O52" s="2"/>
       <c r="P52" s="2"/>
@@ -3643,19 +3647,19 @@
       <c r="AQ52" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="18.75">
-      <c r="A53" s="2"/>
-      <c r="B53" s="2"/>
-      <c r="C53" s="2"/>
-      <c r="D53" s="2"/>
-      <c r="E53" s="2"/>
-      <c r="F53" s="2"/>
-      <c r="G53" s="2"/>
-      <c r="H53" s="2"/>
+      <c r="A53" s="3"/>
+      <c r="B53" s="3"/>
+      <c r="C53" s="3"/>
+      <c r="D53" s="3"/>
+      <c r="E53" s="3"/>
+      <c r="F53" s="3"/>
+      <c r="G53" s="3"/>
+      <c r="H53" s="3"/>
       <c r="I53" s="2"/>
       <c r="J53" s="2"/>
-      <c r="K53" s="2"/>
-      <c r="L53" s="2"/>
-      <c r="M53" s="2"/>
+      <c r="K53" s="3"/>
+      <c r="L53" s="3"/>
+      <c r="M53" s="3"/>
       <c r="N53" s="2"/>
       <c r="O53" s="2"/>
       <c r="P53" s="2"/>
@@ -3688,19 +3692,19 @@
       <c r="AQ53" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="54" customHeight="1" ht="18.75">
-      <c r="A54" s="2"/>
-      <c r="B54" s="2"/>
-      <c r="C54" s="2"/>
-      <c r="D54" s="2"/>
-      <c r="E54" s="2"/>
-      <c r="F54" s="2"/>
-      <c r="G54" s="2"/>
-      <c r="H54" s="2"/>
+      <c r="A54" s="3"/>
+      <c r="B54" s="3"/>
+      <c r="C54" s="3"/>
+      <c r="D54" s="3"/>
+      <c r="E54" s="3"/>
+      <c r="F54" s="3"/>
+      <c r="G54" s="3"/>
+      <c r="H54" s="3"/>
       <c r="I54" s="2"/>
       <c r="J54" s="2"/>
-      <c r="K54" s="2"/>
-      <c r="L54" s="2"/>
-      <c r="M54" s="2"/>
+      <c r="K54" s="3"/>
+      <c r="L54" s="3"/>
+      <c r="M54" s="3"/>
       <c r="N54" s="2"/>
       <c r="O54" s="2"/>
       <c r="P54" s="2"/>
@@ -3733,19 +3737,19 @@
       <c r="AQ54" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18.75">
-      <c r="A55" s="2"/>
-      <c r="B55" s="2"/>
-      <c r="C55" s="2"/>
-      <c r="D55" s="2"/>
-      <c r="E55" s="2"/>
-      <c r="F55" s="2"/>
-      <c r="G55" s="2"/>
-      <c r="H55" s="2"/>
+      <c r="A55" s="3"/>
+      <c r="B55" s="3"/>
+      <c r="C55" s="3"/>
+      <c r="D55" s="3"/>
+      <c r="E55" s="3"/>
+      <c r="F55" s="3"/>
+      <c r="G55" s="3"/>
+      <c r="H55" s="3"/>
       <c r="I55" s="2"/>
       <c r="J55" s="2"/>
-      <c r="K55" s="2"/>
-      <c r="L55" s="2"/>
-      <c r="M55" s="2"/>
+      <c r="K55" s="3"/>
+      <c r="L55" s="3"/>
+      <c r="M55" s="3"/>
       <c r="N55" s="2"/>
       <c r="O55" s="2"/>
       <c r="P55" s="2"/>
@@ -3778,19 +3782,19 @@
       <c r="AQ55" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="56" customHeight="1" ht="18.75">
-      <c r="A56" s="2"/>
-      <c r="B56" s="2"/>
-      <c r="C56" s="2"/>
-      <c r="D56" s="2"/>
-      <c r="E56" s="2"/>
-      <c r="F56" s="2"/>
-      <c r="G56" s="2"/>
-      <c r="H56" s="2"/>
+      <c r="A56" s="3"/>
+      <c r="B56" s="3"/>
+      <c r="C56" s="3"/>
+      <c r="D56" s="3"/>
+      <c r="E56" s="3"/>
+      <c r="F56" s="3"/>
+      <c r="G56" s="3"/>
+      <c r="H56" s="3"/>
       <c r="I56" s="2"/>
       <c r="J56" s="2"/>
-      <c r="K56" s="2"/>
-      <c r="L56" s="2"/>
-      <c r="M56" s="2"/>
+      <c r="K56" s="3"/>
+      <c r="L56" s="3"/>
+      <c r="M56" s="3"/>
       <c r="N56" s="2"/>
       <c r="O56" s="2"/>
       <c r="P56" s="2"/>
@@ -3823,19 +3827,19 @@
       <c r="AQ56" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="57" customHeight="1" ht="18.75">
-      <c r="A57" s="2"/>
-      <c r="B57" s="2"/>
-      <c r="C57" s="2"/>
-      <c r="D57" s="2"/>
-      <c r="E57" s="2"/>
-      <c r="F57" s="2"/>
-      <c r="G57" s="2"/>
-      <c r="H57" s="2"/>
+      <c r="A57" s="3"/>
+      <c r="B57" s="3"/>
+      <c r="C57" s="3"/>
+      <c r="D57" s="3"/>
+      <c r="E57" s="3"/>
+      <c r="F57" s="3"/>
+      <c r="G57" s="3"/>
+      <c r="H57" s="3"/>
       <c r="I57" s="2"/>
       <c r="J57" s="2"/>
-      <c r="K57" s="2"/>
-      <c r="L57" s="2"/>
-      <c r="M57" s="2"/>
+      <c r="K57" s="3"/>
+      <c r="L57" s="3"/>
+      <c r="M57" s="3"/>
       <c r="N57" s="2"/>
       <c r="O57" s="2"/>
       <c r="P57" s="2"/>
@@ -3868,19 +3872,19 @@
       <c r="AQ57" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="18.75">
-      <c r="A58" s="2"/>
-      <c r="B58" s="2"/>
-      <c r="C58" s="2"/>
-      <c r="D58" s="2"/>
-      <c r="E58" s="2"/>
-      <c r="F58" s="2"/>
-      <c r="G58" s="2"/>
-      <c r="H58" s="2"/>
+      <c r="A58" s="3"/>
+      <c r="B58" s="3"/>
+      <c r="C58" s="3"/>
+      <c r="D58" s="3"/>
+      <c r="E58" s="3"/>
+      <c r="F58" s="3"/>
+      <c r="G58" s="3"/>
+      <c r="H58" s="3"/>
       <c r="I58" s="2"/>
       <c r="J58" s="2"/>
-      <c r="K58" s="2"/>
-      <c r="L58" s="2"/>
-      <c r="M58" s="2"/>
+      <c r="K58" s="3"/>
+      <c r="L58" s="3"/>
+      <c r="M58" s="3"/>
       <c r="N58" s="2"/>
       <c r="O58" s="2"/>
       <c r="P58" s="2"/>
@@ -3913,19 +3917,19 @@
       <c r="AQ58" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="18.75">
-      <c r="A59" s="2"/>
-      <c r="B59" s="2"/>
-      <c r="C59" s="2"/>
-      <c r="D59" s="2"/>
-      <c r="E59" s="2"/>
-      <c r="F59" s="2"/>
-      <c r="G59" s="2"/>
-      <c r="H59" s="2"/>
+      <c r="A59" s="3"/>
+      <c r="B59" s="3"/>
+      <c r="C59" s="3"/>
+      <c r="D59" s="3"/>
+      <c r="E59" s="3"/>
+      <c r="F59" s="3"/>
+      <c r="G59" s="3"/>
+      <c r="H59" s="3"/>
       <c r="I59" s="2"/>
       <c r="J59" s="2"/>
-      <c r="K59" s="2"/>
-      <c r="L59" s="2"/>
-      <c r="M59" s="2"/>
+      <c r="K59" s="3"/>
+      <c r="L59" s="3"/>
+      <c r="M59" s="3"/>
       <c r="N59" s="2"/>
       <c r="O59" s="2"/>
       <c r="P59" s="2"/>
@@ -3958,19 +3962,19 @@
       <c r="AQ59" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="18.75">
-      <c r="A60" s="2"/>
-      <c r="B60" s="2"/>
-      <c r="C60" s="2"/>
-      <c r="D60" s="2"/>
-      <c r="E60" s="2"/>
-      <c r="F60" s="2"/>
-      <c r="G60" s="2"/>
-      <c r="H60" s="2"/>
+      <c r="A60" s="3"/>
+      <c r="B60" s="3"/>
+      <c r="C60" s="3"/>
+      <c r="D60" s="3"/>
+      <c r="E60" s="3"/>
+      <c r="F60" s="3"/>
+      <c r="G60" s="3"/>
+      <c r="H60" s="3"/>
       <c r="I60" s="2"/>
       <c r="J60" s="2"/>
-      <c r="K60" s="2"/>
-      <c r="L60" s="2"/>
-      <c r="M60" s="2"/>
+      <c r="K60" s="3"/>
+      <c r="L60" s="3"/>
+      <c r="M60" s="3"/>
       <c r="N60" s="2"/>
       <c r="O60" s="2"/>
       <c r="P60" s="2"/>
@@ -4003,19 +4007,19 @@
       <c r="AQ60" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="18.75">
-      <c r="A61" s="2"/>
-      <c r="B61" s="2"/>
-      <c r="C61" s="2"/>
-      <c r="D61" s="2"/>
-      <c r="E61" s="2"/>
-      <c r="F61" s="2"/>
-      <c r="G61" s="2"/>
-      <c r="H61" s="2"/>
+      <c r="A61" s="3"/>
+      <c r="B61" s="3"/>
+      <c r="C61" s="3"/>
+      <c r="D61" s="3"/>
+      <c r="E61" s="3"/>
+      <c r="F61" s="3"/>
+      <c r="G61" s="3"/>
+      <c r="H61" s="3"/>
       <c r="I61" s="2"/>
       <c r="J61" s="2"/>
-      <c r="K61" s="2"/>
-      <c r="L61" s="2"/>
-      <c r="M61" s="2"/>
+      <c r="K61" s="3"/>
+      <c r="L61" s="3"/>
+      <c r="M61" s="3"/>
       <c r="N61" s="2"/>
       <c r="O61" s="2"/>
       <c r="P61" s="2"/>
@@ -4048,19 +4052,19 @@
       <c r="AQ61" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="18.75">
-      <c r="A62" s="2"/>
-      <c r="B62" s="2"/>
-      <c r="C62" s="2"/>
-      <c r="D62" s="2"/>
-      <c r="E62" s="2"/>
-      <c r="F62" s="2"/>
-      <c r="G62" s="2"/>
-      <c r="H62" s="2"/>
+      <c r="A62" s="3"/>
+      <c r="B62" s="3"/>
+      <c r="C62" s="3"/>
+      <c r="D62" s="3"/>
+      <c r="E62" s="3"/>
+      <c r="F62" s="3"/>
+      <c r="G62" s="3"/>
+      <c r="H62" s="3"/>
       <c r="I62" s="2"/>
       <c r="J62" s="2"/>
-      <c r="K62" s="2"/>
-      <c r="L62" s="2"/>
-      <c r="M62" s="2"/>
+      <c r="K62" s="3"/>
+      <c r="L62" s="3"/>
+      <c r="M62" s="3"/>
       <c r="N62" s="2"/>
       <c r="O62" s="2"/>
       <c r="P62" s="2"/>
@@ -4093,19 +4097,19 @@
       <c r="AQ62" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="63" customHeight="1" ht="18.75">
-      <c r="A63" s="2"/>
-      <c r="B63" s="2"/>
-      <c r="C63" s="2"/>
-      <c r="D63" s="2"/>
-      <c r="E63" s="2"/>
-      <c r="F63" s="2"/>
-      <c r="G63" s="2"/>
-      <c r="H63" s="2"/>
+      <c r="A63" s="3"/>
+      <c r="B63" s="3"/>
+      <c r="C63" s="3"/>
+      <c r="D63" s="3"/>
+      <c r="E63" s="3"/>
+      <c r="F63" s="3"/>
+      <c r="G63" s="3"/>
+      <c r="H63" s="3"/>
       <c r="I63" s="2"/>
       <c r="J63" s="2"/>
-      <c r="K63" s="2"/>
-      <c r="L63" s="2"/>
-      <c r="M63" s="2"/>
+      <c r="K63" s="3"/>
+      <c r="L63" s="3"/>
+      <c r="M63" s="3"/>
       <c r="N63" s="2"/>
       <c r="O63" s="2"/>
       <c r="P63" s="2"/>
@@ -4138,19 +4142,19 @@
       <c r="AQ63" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="18.75">
-      <c r="A64" s="2"/>
-      <c r="B64" s="2"/>
-      <c r="C64" s="2"/>
-      <c r="D64" s="2"/>
-      <c r="E64" s="2"/>
-      <c r="F64" s="2"/>
-      <c r="G64" s="2"/>
-      <c r="H64" s="2"/>
+      <c r="A64" s="3"/>
+      <c r="B64" s="3"/>
+      <c r="C64" s="3"/>
+      <c r="D64" s="3"/>
+      <c r="E64" s="3"/>
+      <c r="F64" s="3"/>
+      <c r="G64" s="3"/>
+      <c r="H64" s="3"/>
       <c r="I64" s="2"/>
       <c r="J64" s="2"/>
-      <c r="K64" s="2"/>
-      <c r="L64" s="2"/>
-      <c r="M64" s="2"/>
+      <c r="K64" s="3"/>
+      <c r="L64" s="3"/>
+      <c r="M64" s="3"/>
       <c r="N64" s="2"/>
       <c r="O64" s="2"/>
       <c r="P64" s="2"/>
@@ -4183,19 +4187,19 @@
       <c r="AQ64" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="65" customHeight="1" ht="18.75">
-      <c r="A65" s="2"/>
-      <c r="B65" s="2"/>
-      <c r="C65" s="2"/>
-      <c r="D65" s="2"/>
-      <c r="E65" s="2"/>
-      <c r="F65" s="2"/>
-      <c r="G65" s="2"/>
-      <c r="H65" s="2"/>
+      <c r="A65" s="3"/>
+      <c r="B65" s="3"/>
+      <c r="C65" s="3"/>
+      <c r="D65" s="3"/>
+      <c r="E65" s="3"/>
+      <c r="F65" s="3"/>
+      <c r="G65" s="3"/>
+      <c r="H65" s="3"/>
       <c r="I65" s="2"/>
       <c r="J65" s="2"/>
-      <c r="K65" s="2"/>
-      <c r="L65" s="2"/>
-      <c r="M65" s="2"/>
+      <c r="K65" s="3"/>
+      <c r="L65" s="3"/>
+      <c r="M65" s="3"/>
       <c r="N65" s="2"/>
       <c r="O65" s="2"/>
       <c r="P65" s="2"/>
@@ -4228,19 +4232,19 @@
       <c r="AQ65" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="66" customHeight="1" ht="18.75">
-      <c r="A66" s="2"/>
-      <c r="B66" s="2"/>
-      <c r="C66" s="2"/>
-      <c r="D66" s="2"/>
-      <c r="E66" s="2"/>
-      <c r="F66" s="2"/>
-      <c r="G66" s="2"/>
-      <c r="H66" s="2"/>
+      <c r="A66" s="3"/>
+      <c r="B66" s="3"/>
+      <c r="C66" s="3"/>
+      <c r="D66" s="3"/>
+      <c r="E66" s="3"/>
+      <c r="F66" s="3"/>
+      <c r="G66" s="3"/>
+      <c r="H66" s="3"/>
       <c r="I66" s="2"/>
       <c r="J66" s="2"/>
-      <c r="K66" s="2"/>
-      <c r="L66" s="2"/>
-      <c r="M66" s="2"/>
+      <c r="K66" s="3"/>
+      <c r="L66" s="3"/>
+      <c r="M66" s="3"/>
       <c r="N66" s="2"/>
       <c r="O66" s="2"/>
       <c r="P66" s="2"/>
@@ -4273,19 +4277,19 @@
       <c r="AQ66" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="18.75">
-      <c r="A67" s="2"/>
-      <c r="B67" s="2"/>
-      <c r="C67" s="2"/>
-      <c r="D67" s="2"/>
-      <c r="E67" s="2"/>
-      <c r="F67" s="2"/>
-      <c r="G67" s="2"/>
-      <c r="H67" s="2"/>
+      <c r="A67" s="3"/>
+      <c r="B67" s="3"/>
+      <c r="C67" s="3"/>
+      <c r="D67" s="3"/>
+      <c r="E67" s="3"/>
+      <c r="F67" s="3"/>
+      <c r="G67" s="3"/>
+      <c r="H67" s="3"/>
       <c r="I67" s="2"/>
       <c r="J67" s="2"/>
-      <c r="K67" s="2"/>
-      <c r="L67" s="2"/>
-      <c r="M67" s="2"/>
+      <c r="K67" s="3"/>
+      <c r="L67" s="3"/>
+      <c r="M67" s="3"/>
       <c r="N67" s="2"/>
       <c r="O67" s="2"/>
       <c r="P67" s="2"/>
@@ -4318,19 +4322,19 @@
       <c r="AQ67" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="18.75">
-      <c r="A68" s="2"/>
-      <c r="B68" s="2"/>
-      <c r="C68" s="2"/>
-      <c r="D68" s="2"/>
-      <c r="E68" s="2"/>
-      <c r="F68" s="2"/>
-      <c r="G68" s="2"/>
-      <c r="H68" s="2"/>
+      <c r="A68" s="3"/>
+      <c r="B68" s="3"/>
+      <c r="C68" s="3"/>
+      <c r="D68" s="3"/>
+      <c r="E68" s="3"/>
+      <c r="F68" s="3"/>
+      <c r="G68" s="3"/>
+      <c r="H68" s="3"/>
       <c r="I68" s="2"/>
       <c r="J68" s="2"/>
-      <c r="K68" s="2"/>
-      <c r="L68" s="2"/>
-      <c r="M68" s="2"/>
+      <c r="K68" s="3"/>
+      <c r="L68" s="3"/>
+      <c r="M68" s="3"/>
       <c r="N68" s="2"/>
       <c r="O68" s="2"/>
       <c r="P68" s="2"/>
@@ -4363,19 +4367,19 @@
       <c r="AQ68" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="18.75">
-      <c r="A69" s="2"/>
-      <c r="B69" s="2"/>
-      <c r="C69" s="2"/>
-      <c r="D69" s="2"/>
-      <c r="E69" s="2"/>
-      <c r="F69" s="2"/>
-      <c r="G69" s="2"/>
-      <c r="H69" s="2"/>
+      <c r="A69" s="3"/>
+      <c r="B69" s="3"/>
+      <c r="C69" s="3"/>
+      <c r="D69" s="3"/>
+      <c r="E69" s="3"/>
+      <c r="F69" s="3"/>
+      <c r="G69" s="3"/>
+      <c r="H69" s="3"/>
       <c r="I69" s="2"/>
       <c r="J69" s="2"/>
-      <c r="K69" s="2"/>
-      <c r="L69" s="2"/>
-      <c r="M69" s="2"/>
+      <c r="K69" s="3"/>
+      <c r="L69" s="3"/>
+      <c r="M69" s="3"/>
       <c r="N69" s="2"/>
       <c r="O69" s="2"/>
       <c r="P69" s="2"/>
@@ -4408,19 +4412,19 @@
       <c r="AQ69" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="18.75">
-      <c r="A70" s="2"/>
-      <c r="B70" s="2"/>
-      <c r="C70" s="2"/>
-      <c r="D70" s="2"/>
-      <c r="E70" s="2"/>
-      <c r="F70" s="2"/>
-      <c r="G70" s="2"/>
-      <c r="H70" s="2"/>
+      <c r="A70" s="3"/>
+      <c r="B70" s="3"/>
+      <c r="C70" s="3"/>
+      <c r="D70" s="3"/>
+      <c r="E70" s="3"/>
+      <c r="F70" s="3"/>
+      <c r="G70" s="3"/>
+      <c r="H70" s="3"/>
       <c r="I70" s="2"/>
       <c r="J70" s="2"/>
-      <c r="K70" s="2"/>
-      <c r="L70" s="2"/>
-      <c r="M70" s="2"/>
+      <c r="K70" s="3"/>
+      <c r="L70" s="3"/>
+      <c r="M70" s="3"/>
       <c r="N70" s="2"/>
       <c r="O70" s="2"/>
       <c r="P70" s="2"/>
@@ -4453,19 +4457,19 @@
       <c r="AQ70" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="71" customHeight="1" ht="18.75">
-      <c r="A71" s="2"/>
-      <c r="B71" s="2"/>
-      <c r="C71" s="2"/>
-      <c r="D71" s="2"/>
-      <c r="E71" s="2"/>
-      <c r="F71" s="2"/>
-      <c r="G71" s="2"/>
-      <c r="H71" s="2"/>
+      <c r="A71" s="3"/>
+      <c r="B71" s="3"/>
+      <c r="C71" s="3"/>
+      <c r="D71" s="3"/>
+      <c r="E71" s="3"/>
+      <c r="F71" s="3"/>
+      <c r="G71" s="3"/>
+      <c r="H71" s="3"/>
       <c r="I71" s="2"/>
       <c r="J71" s="2"/>
-      <c r="K71" s="2"/>
-      <c r="L71" s="2"/>
-      <c r="M71" s="2"/>
+      <c r="K71" s="3"/>
+      <c r="L71" s="3"/>
+      <c r="M71" s="3"/>
       <c r="N71" s="2"/>
       <c r="O71" s="2"/>
       <c r="P71" s="2"/>
@@ -4498,19 +4502,19 @@
       <c r="AQ71" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="72" customHeight="1" ht="18.75">
-      <c r="A72" s="2"/>
-      <c r="B72" s="2"/>
-      <c r="C72" s="2"/>
-      <c r="D72" s="2"/>
-      <c r="E72" s="2"/>
-      <c r="F72" s="2"/>
-      <c r="G72" s="2"/>
-      <c r="H72" s="2"/>
+      <c r="A72" s="3"/>
+      <c r="B72" s="3"/>
+      <c r="C72" s="3"/>
+      <c r="D72" s="3"/>
+      <c r="E72" s="3"/>
+      <c r="F72" s="3"/>
+      <c r="G72" s="3"/>
+      <c r="H72" s="3"/>
       <c r="I72" s="2"/>
       <c r="J72" s="2"/>
-      <c r="K72" s="2"/>
-      <c r="L72" s="2"/>
-      <c r="M72" s="2"/>
+      <c r="K72" s="3"/>
+      <c r="L72" s="3"/>
+      <c r="M72" s="3"/>
       <c r="N72" s="2"/>
       <c r="O72" s="2"/>
       <c r="P72" s="2"/>
@@ -4543,19 +4547,19 @@
       <c r="AQ72" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="73" customHeight="1" ht="18.75">
-      <c r="A73" s="2"/>
-      <c r="B73" s="2"/>
-      <c r="C73" s="2"/>
-      <c r="D73" s="2"/>
-      <c r="E73" s="2"/>
-      <c r="F73" s="2"/>
-      <c r="G73" s="2"/>
-      <c r="H73" s="2"/>
+      <c r="A73" s="3"/>
+      <c r="B73" s="3"/>
+      <c r="C73" s="3"/>
+      <c r="D73" s="3"/>
+      <c r="E73" s="3"/>
+      <c r="F73" s="3"/>
+      <c r="G73" s="3"/>
+      <c r="H73" s="3"/>
       <c r="I73" s="2"/>
       <c r="J73" s="2"/>
-      <c r="K73" s="2"/>
-      <c r="L73" s="2"/>
-      <c r="M73" s="2"/>
+      <c r="K73" s="3"/>
+      <c r="L73" s="3"/>
+      <c r="M73" s="3"/>
       <c r="N73" s="2"/>
       <c r="O73" s="2"/>
       <c r="P73" s="2"/>
@@ -4588,19 +4592,19 @@
       <c r="AQ73" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="74" customHeight="1" ht="18.75">
-      <c r="A74" s="2"/>
-      <c r="B74" s="2"/>
-      <c r="C74" s="2"/>
-      <c r="D74" s="2"/>
-      <c r="E74" s="2"/>
-      <c r="F74" s="2"/>
-      <c r="G74" s="2"/>
-      <c r="H74" s="2"/>
+      <c r="A74" s="3"/>
+      <c r="B74" s="3"/>
+      <c r="C74" s="3"/>
+      <c r="D74" s="3"/>
+      <c r="E74" s="3"/>
+      <c r="F74" s="3"/>
+      <c r="G74" s="3"/>
+      <c r="H74" s="3"/>
       <c r="I74" s="2"/>
       <c r="J74" s="2"/>
-      <c r="K74" s="2"/>
-      <c r="L74" s="2"/>
-      <c r="M74" s="2"/>
+      <c r="K74" s="3"/>
+      <c r="L74" s="3"/>
+      <c r="M74" s="3"/>
       <c r="N74" s="2"/>
       <c r="O74" s="2"/>
       <c r="P74" s="2"/>
@@ -4633,19 +4637,19 @@
       <c r="AQ74" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="75" customHeight="1" ht="18.75">
-      <c r="A75" s="2"/>
-      <c r="B75" s="2"/>
-      <c r="C75" s="2"/>
-      <c r="D75" s="2"/>
-      <c r="E75" s="2"/>
-      <c r="F75" s="2"/>
-      <c r="G75" s="2"/>
-      <c r="H75" s="2"/>
+      <c r="A75" s="3"/>
+      <c r="B75" s="3"/>
+      <c r="C75" s="3"/>
+      <c r="D75" s="3"/>
+      <c r="E75" s="3"/>
+      <c r="F75" s="3"/>
+      <c r="G75" s="3"/>
+      <c r="H75" s="3"/>
       <c r="I75" s="2"/>
       <c r="J75" s="2"/>
-      <c r="K75" s="2"/>
-      <c r="L75" s="2"/>
-      <c r="M75" s="2"/>
+      <c r="K75" s="3"/>
+      <c r="L75" s="3"/>
+      <c r="M75" s="3"/>
       <c r="N75" s="2"/>
       <c r="O75" s="2"/>
       <c r="P75" s="2"/>
@@ -4678,19 +4682,19 @@
       <c r="AQ75" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="76" customHeight="1" ht="18.75">
-      <c r="A76" s="2"/>
-      <c r="B76" s="2"/>
-      <c r="C76" s="2"/>
-      <c r="D76" s="2"/>
-      <c r="E76" s="2"/>
-      <c r="F76" s="2"/>
-      <c r="G76" s="2"/>
-      <c r="H76" s="2"/>
+      <c r="A76" s="3"/>
+      <c r="B76" s="3"/>
+      <c r="C76" s="3"/>
+      <c r="D76" s="3"/>
+      <c r="E76" s="3"/>
+      <c r="F76" s="3"/>
+      <c r="G76" s="3"/>
+      <c r="H76" s="3"/>
       <c r="I76" s="2"/>
       <c r="J76" s="2"/>
-      <c r="K76" s="2"/>
-      <c r="L76" s="2"/>
-      <c r="M76" s="2"/>
+      <c r="K76" s="3"/>
+      <c r="L76" s="3"/>
+      <c r="M76" s="3"/>
       <c r="N76" s="2"/>
       <c r="O76" s="2"/>
       <c r="P76" s="2"/>
@@ -4723,19 +4727,19 @@
       <c r="AQ76" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="77" customHeight="1" ht="18.75">
-      <c r="A77" s="2"/>
-      <c r="B77" s="2"/>
-      <c r="C77" s="2"/>
-      <c r="D77" s="2"/>
-      <c r="E77" s="2"/>
-      <c r="F77" s="2"/>
-      <c r="G77" s="2"/>
-      <c r="H77" s="2"/>
+      <c r="A77" s="3"/>
+      <c r="B77" s="3"/>
+      <c r="C77" s="3"/>
+      <c r="D77" s="3"/>
+      <c r="E77" s="3"/>
+      <c r="F77" s="3"/>
+      <c r="G77" s="3"/>
+      <c r="H77" s="3"/>
       <c r="I77" s="2"/>
       <c r="J77" s="2"/>
-      <c r="K77" s="2"/>
-      <c r="L77" s="2"/>
-      <c r="M77" s="2"/>
+      <c r="K77" s="3"/>
+      <c r="L77" s="3"/>
+      <c r="M77" s="3"/>
       <c r="N77" s="2"/>
       <c r="O77" s="2"/>
       <c r="P77" s="2"/>

</xml_diff>

<commit_message>
Correction des descriptions + correction du css
</commit_message>
<xml_diff>
--- a/docs/SSZ_TableauDeSynthese.xlsx
+++ b/docs/SSZ_TableauDeSynthese.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="47">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -161,6 +161,9 @@
     <t>Stage dans l'entreprise Sateb</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t>Projet application type ocs inventory</t>
   </si>
   <si>
@@ -197,6 +200,12 @@
       <family val="2"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
       <b/>
       <sz val="18"/>
       <color rgb="FF000000"/>
@@ -222,12 +231,6 @@
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
@@ -664,145 +667,154 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="52">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="4" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="5" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="6" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="7" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="8" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="9" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="10" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="8" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="11" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="12" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="13" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="14" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="15" applyBorder="1" fontId="5" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="16" applyBorder="1" fontId="6" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="17" applyBorder="1" fontId="6" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="18" applyBorder="1" fontId="6" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="19" applyBorder="1" fontId="5" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="20" applyBorder="1" fontId="6" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="21" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="22" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="23" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="17" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="18" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="24" applyBorder="1" fontId="9" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="25" applyBorder="1" fontId="9" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="25" applyBorder="1" fontId="10" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="25" applyBorder="1" fontId="11" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="26" applyBorder="1" fontId="11" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="24" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="25" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="26" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="25" applyBorder="1" fontId="11" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="26" applyBorder="1" fontId="11" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="27" applyBorder="1" fontId="9" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="28" applyBorder="1" fontId="9" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="28" applyBorder="1" fontId="11" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="29" applyBorder="1" fontId="11" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="9" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="9" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="11" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="4" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="5" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="6" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="7" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="8" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="9" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="10" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="8" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="11" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="12" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="13" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="14" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="15" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="16" applyBorder="1" fontId="5" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="17" applyBorder="1" fontId="5" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="18" applyBorder="1" fontId="5" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="6" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="19" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="20" applyBorder="1" fontId="5" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="21" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="22" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="23" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="17" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="18" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="24" applyBorder="1" fontId="9" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="25" applyBorder="1" fontId="9" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="25" applyBorder="1" fontId="10" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="25" applyBorder="1" fontId="11" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="26" applyBorder="1" fontId="11" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="24" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="25" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="26" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="27" applyBorder="1" fontId="9" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="28" applyBorder="1" fontId="9" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="28" applyBorder="1" fontId="11" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="29" applyBorder="1" fontId="11" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="9" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="9" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="11" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
@@ -1115,49 +1127,49 @@
   <dimension ref="A1:AQ77"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="47" width="70.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="47" width="10.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="47" width="18.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="47" width="18.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="47" width="18.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="47" width="18.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="47" width="18.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="47" width="18.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="47" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="47" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="47" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="23" max="23" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="24" max="24" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="25" max="25" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="26" max="26" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="27" max="27" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="28" max="28" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="29" max="29" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="30" max="30" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="31" max="31" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="32" max="32" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="33" max="33" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="34" max="34" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="35" max="35" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="36" max="36" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="37" max="37" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="38" max="38" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="39" max="39" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="40" max="40" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="41" max="41" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="42" max="42" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="43" max="43" style="48" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="50" width="70.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="50" width="10.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="50" width="18.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="50" width="18.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="50" width="18.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="50" width="18.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="50" width="18.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="50" width="18.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="51" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="51" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="50" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="50" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="50" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="51" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="51" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="51" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="51" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="51" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="51" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="51" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="51" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="51" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="23" max="23" style="51" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="24" max="24" style="51" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="25" max="25" style="51" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="26" max="26" style="51" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="27" max="27" style="51" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="28" max="28" style="51" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="29" max="29" style="51" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="30" max="30" style="51" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="31" max="31" style="51" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="32" max="32" style="51" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="33" max="33" style="51" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="34" max="34" style="51" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="35" max="35" style="51" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="36" max="36" style="51" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="37" max="37" style="51" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="38" max="38" style="51" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="39" max="39" style="51" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="40" max="40" style="51" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="41" max="41" style="51" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="42" max="42" style="51" width="11.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="43" max="43" style="51" width="11.43357142857143" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="29.25">
@@ -2276,8 +2288,8 @@
       <c r="E23" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="F23" s="35" t="s">
-        <v>26</v>
+      <c r="F23" s="40" t="s">
+        <v>41</v>
       </c>
       <c r="G23" s="35"/>
       <c r="H23" s="36"/>
@@ -2319,7 +2331,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
       <c r="A24" s="32" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B24" s="33"/>
       <c r="C24" s="35"/>
@@ -2364,7 +2376,7 @@
       <c r="AP24" s="2"/>
       <c r="AQ24" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="39.95">
+    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
       <c r="A25" s="32"/>
       <c r="B25" s="33"/>
       <c r="C25" s="35"/>
@@ -2409,9 +2421,9 @@
       <c r="AP25" s="2"/>
       <c r="AQ25" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="22.5">
       <c r="A26" s="37" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B26" s="38"/>
       <c r="C26" s="38"/>
@@ -2456,9 +2468,9 @@
       <c r="AP26" s="2"/>
       <c r="AQ26" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="39.95">
+    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
       <c r="A27" s="32" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B27" s="33"/>
       <c r="C27" s="35"/>
@@ -2472,8 +2484,8 @@
         <v>26</v>
       </c>
       <c r="G27" s="35"/>
-      <c r="H27" s="36" t="s">
-        <v>26</v>
+      <c r="H27" s="41" t="s">
+        <v>41</v>
       </c>
       <c r="I27" s="2"/>
       <c r="J27" s="2"/>
@@ -2511,9 +2523,9 @@
       <c r="AP27" s="2"/>
       <c r="AQ27" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="39.95">
+    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
       <c r="A28" s="32" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B28" s="33"/>
       <c r="C28" s="35"/>
@@ -2562,9 +2574,9 @@
       <c r="AP28" s="2"/>
       <c r="AQ28" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="39.95">
+    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75">
       <c r="A29" s="32" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B29" s="33"/>
       <c r="C29" s="35"/>
@@ -2611,15 +2623,15 @@
       <c r="AP29" s="2"/>
       <c r="AQ29" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="39.95">
-      <c r="A30" s="40"/>
-      <c r="B30" s="41"/>
-      <c r="C30" s="42"/>
-      <c r="D30" s="42"/>
-      <c r="E30" s="42"/>
-      <c r="F30" s="42"/>
-      <c r="G30" s="42"/>
-      <c r="H30" s="43"/>
+    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="19.5">
+      <c r="A30" s="42"/>
+      <c r="B30" s="43"/>
+      <c r="C30" s="44"/>
+      <c r="D30" s="44"/>
+      <c r="E30" s="44"/>
+      <c r="F30" s="44"/>
+      <c r="G30" s="44"/>
+      <c r="H30" s="45"/>
       <c r="I30" s="2"/>
       <c r="J30" s="2"/>
       <c r="K30" s="3"/>
@@ -2656,15 +2668,15 @@
       <c r="AP30" s="2"/>
       <c r="AQ30" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75">
-      <c r="A31" s="44"/>
-      <c r="B31" s="45"/>
-      <c r="C31" s="46"/>
-      <c r="D31" s="46"/>
-      <c r="E31" s="46"/>
-      <c r="F31" s="46"/>
-      <c r="G31" s="46"/>
-      <c r="H31" s="46"/>
+    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="19.5">
+      <c r="A31" s="46"/>
+      <c r="B31" s="47"/>
+      <c r="C31" s="48"/>
+      <c r="D31" s="48"/>
+      <c r="E31" s="48"/>
+      <c r="F31" s="48"/>
+      <c r="G31" s="48"/>
+      <c r="H31" s="48"/>
       <c r="I31" s="2"/>
       <c r="J31" s="2"/>
       <c r="K31" s="3"/>
@@ -2701,20 +2713,20 @@
       <c r="AP31" s="2"/>
       <c r="AQ31" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
-      <c r="A32" s="3"/>
-      <c r="B32" s="3"/>
-      <c r="C32" s="3"/>
-      <c r="D32" s="3"/>
-      <c r="E32" s="3"/>
-      <c r="F32" s="3"/>
-      <c r="G32" s="3"/>
-      <c r="H32" s="3"/>
+    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A32" s="49"/>
+      <c r="B32" s="49"/>
+      <c r="C32" s="49"/>
+      <c r="D32" s="49"/>
+      <c r="E32" s="49"/>
+      <c r="F32" s="49"/>
+      <c r="G32" s="49"/>
+      <c r="H32" s="49"/>
       <c r="I32" s="2"/>
       <c r="J32" s="2"/>
-      <c r="K32" s="3"/>
-      <c r="L32" s="3"/>
-      <c r="M32" s="3"/>
+      <c r="K32" s="49"/>
+      <c r="L32" s="49"/>
+      <c r="M32" s="49"/>
       <c r="N32" s="2"/>
       <c r="O32" s="2"/>
       <c r="P32" s="2"/>
@@ -2746,20 +2758,20 @@
       <c r="AP32" s="2"/>
       <c r="AQ32" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75">
-      <c r="A33" s="3"/>
-      <c r="B33" s="3"/>
-      <c r="C33" s="3"/>
-      <c r="D33" s="3"/>
-      <c r="E33" s="3"/>
-      <c r="F33" s="3"/>
-      <c r="G33" s="3"/>
-      <c r="H33" s="3"/>
+    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A33" s="49"/>
+      <c r="B33" s="49"/>
+      <c r="C33" s="49"/>
+      <c r="D33" s="49"/>
+      <c r="E33" s="49"/>
+      <c r="F33" s="49"/>
+      <c r="G33" s="49"/>
+      <c r="H33" s="49"/>
       <c r="I33" s="2"/>
       <c r="J33" s="2"/>
-      <c r="K33" s="3"/>
-      <c r="L33" s="3"/>
-      <c r="M33" s="3"/>
+      <c r="K33" s="49"/>
+      <c r="L33" s="49"/>
+      <c r="M33" s="49"/>
       <c r="N33" s="2"/>
       <c r="O33" s="2"/>
       <c r="P33" s="2"/>
@@ -2791,20 +2803,20 @@
       <c r="AP33" s="2"/>
       <c r="AQ33" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
-      <c r="A34" s="3"/>
-      <c r="B34" s="3"/>
-      <c r="C34" s="3"/>
-      <c r="D34" s="3"/>
-      <c r="E34" s="3"/>
-      <c r="F34" s="3"/>
-      <c r="G34" s="3"/>
-      <c r="H34" s="3"/>
+    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A34" s="49"/>
+      <c r="B34" s="49"/>
+      <c r="C34" s="49"/>
+      <c r="D34" s="49"/>
+      <c r="E34" s="49"/>
+      <c r="F34" s="49"/>
+      <c r="G34" s="49"/>
+      <c r="H34" s="49"/>
       <c r="I34" s="2"/>
       <c r="J34" s="2"/>
-      <c r="K34" s="3"/>
-      <c r="L34" s="3"/>
-      <c r="M34" s="3"/>
+      <c r="K34" s="49"/>
+      <c r="L34" s="49"/>
+      <c r="M34" s="49"/>
       <c r="N34" s="2"/>
       <c r="O34" s="2"/>
       <c r="P34" s="2"/>
@@ -2836,20 +2848,20 @@
       <c r="AP34" s="2"/>
       <c r="AQ34" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75">
-      <c r="A35" s="3"/>
-      <c r="B35" s="3"/>
-      <c r="C35" s="3"/>
-      <c r="D35" s="3"/>
-      <c r="E35" s="3"/>
-      <c r="F35" s="3"/>
-      <c r="G35" s="3"/>
-      <c r="H35" s="3"/>
+    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A35" s="49"/>
+      <c r="B35" s="49"/>
+      <c r="C35" s="49"/>
+      <c r="D35" s="49"/>
+      <c r="E35" s="49"/>
+      <c r="F35" s="49"/>
+      <c r="G35" s="49"/>
+      <c r="H35" s="49"/>
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
-      <c r="K35" s="3"/>
-      <c r="L35" s="3"/>
-      <c r="M35" s="3"/>
+      <c r="K35" s="49"/>
+      <c r="L35" s="49"/>
+      <c r="M35" s="49"/>
       <c r="N35" s="2"/>
       <c r="O35" s="2"/>
       <c r="P35" s="2"/>
@@ -2881,20 +2893,20 @@
       <c r="AP35" s="2"/>
       <c r="AQ35" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75">
-      <c r="A36" s="3"/>
-      <c r="B36" s="3"/>
-      <c r="C36" s="3"/>
-      <c r="D36" s="3"/>
-      <c r="E36" s="3"/>
-      <c r="F36" s="3"/>
-      <c r="G36" s="3"/>
-      <c r="H36" s="3"/>
+    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A36" s="49"/>
+      <c r="B36" s="49"/>
+      <c r="C36" s="49"/>
+      <c r="D36" s="49"/>
+      <c r="E36" s="49"/>
+      <c r="F36" s="49"/>
+      <c r="G36" s="49"/>
+      <c r="H36" s="49"/>
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
-      <c r="K36" s="3"/>
-      <c r="L36" s="3"/>
-      <c r="M36" s="3"/>
+      <c r="K36" s="49"/>
+      <c r="L36" s="49"/>
+      <c r="M36" s="49"/>
       <c r="N36" s="2"/>
       <c r="O36" s="2"/>
       <c r="P36" s="2"/>
@@ -2926,20 +2938,20 @@
       <c r="AP36" s="2"/>
       <c r="AQ36" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75">
-      <c r="A37" s="3"/>
-      <c r="B37" s="3"/>
-      <c r="C37" s="3"/>
-      <c r="D37" s="3"/>
-      <c r="E37" s="3"/>
-      <c r="F37" s="3"/>
-      <c r="G37" s="3"/>
-      <c r="H37" s="3"/>
+    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A37" s="49"/>
+      <c r="B37" s="49"/>
+      <c r="C37" s="49"/>
+      <c r="D37" s="49"/>
+      <c r="E37" s="49"/>
+      <c r="F37" s="49"/>
+      <c r="G37" s="49"/>
+      <c r="H37" s="49"/>
       <c r="I37" s="2"/>
       <c r="J37" s="2"/>
-      <c r="K37" s="3"/>
-      <c r="L37" s="3"/>
-      <c r="M37" s="3"/>
+      <c r="K37" s="49"/>
+      <c r="L37" s="49"/>
+      <c r="M37" s="49"/>
       <c r="N37" s="2"/>
       <c r="O37" s="2"/>
       <c r="P37" s="2"/>
@@ -2971,20 +2983,20 @@
       <c r="AP37" s="2"/>
       <c r="AQ37" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18.75">
-      <c r="A38" s="3"/>
-      <c r="B38" s="3"/>
-      <c r="C38" s="3"/>
-      <c r="D38" s="3"/>
-      <c r="E38" s="3"/>
-      <c r="F38" s="3"/>
-      <c r="G38" s="3"/>
-      <c r="H38" s="3"/>
+    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A38" s="49"/>
+      <c r="B38" s="49"/>
+      <c r="C38" s="49"/>
+      <c r="D38" s="49"/>
+      <c r="E38" s="49"/>
+      <c r="F38" s="49"/>
+      <c r="G38" s="49"/>
+      <c r="H38" s="49"/>
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
-      <c r="K38" s="3"/>
-      <c r="L38" s="3"/>
-      <c r="M38" s="3"/>
+      <c r="K38" s="49"/>
+      <c r="L38" s="49"/>
+      <c r="M38" s="49"/>
       <c r="N38" s="2"/>
       <c r="O38" s="2"/>
       <c r="P38" s="2"/>
@@ -3016,20 +3028,20 @@
       <c r="AP38" s="2"/>
       <c r="AQ38" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18.75">
-      <c r="A39" s="3"/>
-      <c r="B39" s="3"/>
-      <c r="C39" s="3"/>
-      <c r="D39" s="3"/>
-      <c r="E39" s="3"/>
-      <c r="F39" s="3"/>
-      <c r="G39" s="3"/>
-      <c r="H39" s="3"/>
+    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A39" s="49"/>
+      <c r="B39" s="49"/>
+      <c r="C39" s="49"/>
+      <c r="D39" s="49"/>
+      <c r="E39" s="49"/>
+      <c r="F39" s="49"/>
+      <c r="G39" s="49"/>
+      <c r="H39" s="49"/>
       <c r="I39" s="2"/>
       <c r="J39" s="2"/>
-      <c r="K39" s="3"/>
-      <c r="L39" s="3"/>
-      <c r="M39" s="3"/>
+      <c r="K39" s="49"/>
+      <c r="L39" s="49"/>
+      <c r="M39" s="49"/>
       <c r="N39" s="2"/>
       <c r="O39" s="2"/>
       <c r="P39" s="2"/>
@@ -3061,20 +3073,20 @@
       <c r="AP39" s="2"/>
       <c r="AQ39" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18.75">
-      <c r="A40" s="3"/>
-      <c r="B40" s="3"/>
-      <c r="C40" s="3"/>
-      <c r="D40" s="3"/>
-      <c r="E40" s="3"/>
-      <c r="F40" s="3"/>
-      <c r="G40" s="3"/>
-      <c r="H40" s="3"/>
+    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A40" s="49"/>
+      <c r="B40" s="49"/>
+      <c r="C40" s="49"/>
+      <c r="D40" s="49"/>
+      <c r="E40" s="49"/>
+      <c r="F40" s="49"/>
+      <c r="G40" s="49"/>
+      <c r="H40" s="49"/>
       <c r="I40" s="2"/>
       <c r="J40" s="2"/>
-      <c r="K40" s="3"/>
-      <c r="L40" s="3"/>
-      <c r="M40" s="3"/>
+      <c r="K40" s="49"/>
+      <c r="L40" s="49"/>
+      <c r="M40" s="49"/>
       <c r="N40" s="2"/>
       <c r="O40" s="2"/>
       <c r="P40" s="2"/>
@@ -3106,20 +3118,20 @@
       <c r="AP40" s="2"/>
       <c r="AQ40" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18.75">
-      <c r="A41" s="3"/>
-      <c r="B41" s="3"/>
-      <c r="C41" s="3"/>
-      <c r="D41" s="3"/>
-      <c r="E41" s="3"/>
-      <c r="F41" s="3"/>
-      <c r="G41" s="3"/>
-      <c r="H41" s="3"/>
+    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A41" s="49"/>
+      <c r="B41" s="49"/>
+      <c r="C41" s="49"/>
+      <c r="D41" s="49"/>
+      <c r="E41" s="49"/>
+      <c r="F41" s="49"/>
+      <c r="G41" s="49"/>
+      <c r="H41" s="49"/>
       <c r="I41" s="2"/>
       <c r="J41" s="2"/>
-      <c r="K41" s="3"/>
-      <c r="L41" s="3"/>
-      <c r="M41" s="3"/>
+      <c r="K41" s="49"/>
+      <c r="L41" s="49"/>
+      <c r="M41" s="49"/>
       <c r="N41" s="2"/>
       <c r="O41" s="2"/>
       <c r="P41" s="2"/>
@@ -3151,20 +3163,20 @@
       <c r="AP41" s="2"/>
       <c r="AQ41" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18.75">
-      <c r="A42" s="3"/>
-      <c r="B42" s="3"/>
-      <c r="C42" s="3"/>
-      <c r="D42" s="3"/>
-      <c r="E42" s="3"/>
-      <c r="F42" s="3"/>
-      <c r="G42" s="3"/>
-      <c r="H42" s="3"/>
+    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A42" s="49"/>
+      <c r="B42" s="49"/>
+      <c r="C42" s="49"/>
+      <c r="D42" s="49"/>
+      <c r="E42" s="49"/>
+      <c r="F42" s="49"/>
+      <c r="G42" s="49"/>
+      <c r="H42" s="49"/>
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
-      <c r="K42" s="3"/>
-      <c r="L42" s="3"/>
-      <c r="M42" s="3"/>
+      <c r="K42" s="49"/>
+      <c r="L42" s="49"/>
+      <c r="M42" s="49"/>
       <c r="N42" s="2"/>
       <c r="O42" s="2"/>
       <c r="P42" s="2"/>
@@ -3196,20 +3208,20 @@
       <c r="AP42" s="2"/>
       <c r="AQ42" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="18.75">
-      <c r="A43" s="3"/>
-      <c r="B43" s="3"/>
-      <c r="C43" s="3"/>
-      <c r="D43" s="3"/>
-      <c r="E43" s="3"/>
-      <c r="F43" s="3"/>
-      <c r="G43" s="3"/>
-      <c r="H43" s="3"/>
+    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A43" s="49"/>
+      <c r="B43" s="49"/>
+      <c r="C43" s="49"/>
+      <c r="D43" s="49"/>
+      <c r="E43" s="49"/>
+      <c r="F43" s="49"/>
+      <c r="G43" s="49"/>
+      <c r="H43" s="49"/>
       <c r="I43" s="2"/>
       <c r="J43" s="2"/>
-      <c r="K43" s="3"/>
-      <c r="L43" s="3"/>
-      <c r="M43" s="3"/>
+      <c r="K43" s="49"/>
+      <c r="L43" s="49"/>
+      <c r="M43" s="49"/>
       <c r="N43" s="2"/>
       <c r="O43" s="2"/>
       <c r="P43" s="2"/>
@@ -3241,20 +3253,20 @@
       <c r="AP43" s="2"/>
       <c r="AQ43" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="18.75">
-      <c r="A44" s="3"/>
-      <c r="B44" s="3"/>
-      <c r="C44" s="3"/>
-      <c r="D44" s="3"/>
-      <c r="E44" s="3"/>
-      <c r="F44" s="3"/>
-      <c r="G44" s="3"/>
-      <c r="H44" s="3"/>
+    <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A44" s="49"/>
+      <c r="B44" s="49"/>
+      <c r="C44" s="49"/>
+      <c r="D44" s="49"/>
+      <c r="E44" s="49"/>
+      <c r="F44" s="49"/>
+      <c r="G44" s="49"/>
+      <c r="H44" s="49"/>
       <c r="I44" s="2"/>
       <c r="J44" s="2"/>
-      <c r="K44" s="3"/>
-      <c r="L44" s="3"/>
-      <c r="M44" s="3"/>
+      <c r="K44" s="49"/>
+      <c r="L44" s="49"/>
+      <c r="M44" s="49"/>
       <c r="N44" s="2"/>
       <c r="O44" s="2"/>
       <c r="P44" s="2"/>
@@ -3286,20 +3298,20 @@
       <c r="AP44" s="2"/>
       <c r="AQ44" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="18.75">
-      <c r="A45" s="3"/>
-      <c r="B45" s="3"/>
-      <c r="C45" s="3"/>
-      <c r="D45" s="3"/>
-      <c r="E45" s="3"/>
-      <c r="F45" s="3"/>
-      <c r="G45" s="3"/>
-      <c r="H45" s="3"/>
+    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A45" s="49"/>
+      <c r="B45" s="49"/>
+      <c r="C45" s="49"/>
+      <c r="D45" s="49"/>
+      <c r="E45" s="49"/>
+      <c r="F45" s="49"/>
+      <c r="G45" s="49"/>
+      <c r="H45" s="49"/>
       <c r="I45" s="2"/>
       <c r="J45" s="2"/>
-      <c r="K45" s="3"/>
-      <c r="L45" s="3"/>
-      <c r="M45" s="3"/>
+      <c r="K45" s="49"/>
+      <c r="L45" s="49"/>
+      <c r="M45" s="49"/>
       <c r="N45" s="2"/>
       <c r="O45" s="2"/>
       <c r="P45" s="2"/>
@@ -3331,20 +3343,20 @@
       <c r="AP45" s="2"/>
       <c r="AQ45" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="18.75">
-      <c r="A46" s="3"/>
-      <c r="B46" s="3"/>
-      <c r="C46" s="3"/>
-      <c r="D46" s="3"/>
-      <c r="E46" s="3"/>
-      <c r="F46" s="3"/>
-      <c r="G46" s="3"/>
-      <c r="H46" s="3"/>
+    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A46" s="49"/>
+      <c r="B46" s="49"/>
+      <c r="C46" s="49"/>
+      <c r="D46" s="49"/>
+      <c r="E46" s="49"/>
+      <c r="F46" s="49"/>
+      <c r="G46" s="49"/>
+      <c r="H46" s="49"/>
       <c r="I46" s="2"/>
       <c r="J46" s="2"/>
-      <c r="K46" s="3"/>
-      <c r="L46" s="3"/>
-      <c r="M46" s="3"/>
+      <c r="K46" s="49"/>
+      <c r="L46" s="49"/>
+      <c r="M46" s="49"/>
       <c r="N46" s="2"/>
       <c r="O46" s="2"/>
       <c r="P46" s="2"/>
@@ -3376,20 +3388,20 @@
       <c r="AP46" s="2"/>
       <c r="AQ46" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="18.75">
-      <c r="A47" s="3"/>
-      <c r="B47" s="3"/>
-      <c r="C47" s="3"/>
-      <c r="D47" s="3"/>
-      <c r="E47" s="3"/>
-      <c r="F47" s="3"/>
-      <c r="G47" s="3"/>
-      <c r="H47" s="3"/>
+    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A47" s="49"/>
+      <c r="B47" s="49"/>
+      <c r="C47" s="49"/>
+      <c r="D47" s="49"/>
+      <c r="E47" s="49"/>
+      <c r="F47" s="49"/>
+      <c r="G47" s="49"/>
+      <c r="H47" s="49"/>
       <c r="I47" s="2"/>
       <c r="J47" s="2"/>
-      <c r="K47" s="3"/>
-      <c r="L47" s="3"/>
-      <c r="M47" s="3"/>
+      <c r="K47" s="49"/>
+      <c r="L47" s="49"/>
+      <c r="M47" s="49"/>
       <c r="N47" s="2"/>
       <c r="O47" s="2"/>
       <c r="P47" s="2"/>
@@ -3421,20 +3433,20 @@
       <c r="AP47" s="2"/>
       <c r="AQ47" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="18.75">
-      <c r="A48" s="3"/>
-      <c r="B48" s="3"/>
-      <c r="C48" s="3"/>
-      <c r="D48" s="3"/>
-      <c r="E48" s="3"/>
-      <c r="F48" s="3"/>
-      <c r="G48" s="3"/>
-      <c r="H48" s="3"/>
+    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A48" s="49"/>
+      <c r="B48" s="49"/>
+      <c r="C48" s="49"/>
+      <c r="D48" s="49"/>
+      <c r="E48" s="49"/>
+      <c r="F48" s="49"/>
+      <c r="G48" s="49"/>
+      <c r="H48" s="49"/>
       <c r="I48" s="2"/>
       <c r="J48" s="2"/>
-      <c r="K48" s="3"/>
-      <c r="L48" s="3"/>
-      <c r="M48" s="3"/>
+      <c r="K48" s="49"/>
+      <c r="L48" s="49"/>
+      <c r="M48" s="49"/>
       <c r="N48" s="2"/>
       <c r="O48" s="2"/>
       <c r="P48" s="2"/>
@@ -3466,20 +3478,20 @@
       <c r="AP48" s="2"/>
       <c r="AQ48" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="18.75">
-      <c r="A49" s="3"/>
-      <c r="B49" s="3"/>
-      <c r="C49" s="3"/>
-      <c r="D49" s="3"/>
-      <c r="E49" s="3"/>
-      <c r="F49" s="3"/>
-      <c r="G49" s="3"/>
-      <c r="H49" s="3"/>
+    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A49" s="49"/>
+      <c r="B49" s="49"/>
+      <c r="C49" s="49"/>
+      <c r="D49" s="49"/>
+      <c r="E49" s="49"/>
+      <c r="F49" s="49"/>
+      <c r="G49" s="49"/>
+      <c r="H49" s="49"/>
       <c r="I49" s="2"/>
       <c r="J49" s="2"/>
-      <c r="K49" s="3"/>
-      <c r="L49" s="3"/>
-      <c r="M49" s="3"/>
+      <c r="K49" s="49"/>
+      <c r="L49" s="49"/>
+      <c r="M49" s="49"/>
       <c r="N49" s="2"/>
       <c r="O49" s="2"/>
       <c r="P49" s="2"/>
@@ -3511,20 +3523,20 @@
       <c r="AP49" s="2"/>
       <c r="AQ49" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="18.75">
-      <c r="A50" s="3"/>
-      <c r="B50" s="3"/>
-      <c r="C50" s="3"/>
-      <c r="D50" s="3"/>
-      <c r="E50" s="3"/>
-      <c r="F50" s="3"/>
-      <c r="G50" s="3"/>
-      <c r="H50" s="3"/>
+    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A50" s="49"/>
+      <c r="B50" s="49"/>
+      <c r="C50" s="49"/>
+      <c r="D50" s="49"/>
+      <c r="E50" s="49"/>
+      <c r="F50" s="49"/>
+      <c r="G50" s="49"/>
+      <c r="H50" s="49"/>
       <c r="I50" s="2"/>
       <c r="J50" s="2"/>
-      <c r="K50" s="3"/>
-      <c r="L50" s="3"/>
-      <c r="M50" s="3"/>
+      <c r="K50" s="49"/>
+      <c r="L50" s="49"/>
+      <c r="M50" s="49"/>
       <c r="N50" s="2"/>
       <c r="O50" s="2"/>
       <c r="P50" s="2"/>
@@ -3556,20 +3568,20 @@
       <c r="AP50" s="2"/>
       <c r="AQ50" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="18.75">
-      <c r="A51" s="3"/>
-      <c r="B51" s="3"/>
-      <c r="C51" s="3"/>
-      <c r="D51" s="3"/>
-      <c r="E51" s="3"/>
-      <c r="F51" s="3"/>
-      <c r="G51" s="3"/>
-      <c r="H51" s="3"/>
+    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A51" s="49"/>
+      <c r="B51" s="49"/>
+      <c r="C51" s="49"/>
+      <c r="D51" s="49"/>
+      <c r="E51" s="49"/>
+      <c r="F51" s="49"/>
+      <c r="G51" s="49"/>
+      <c r="H51" s="49"/>
       <c r="I51" s="2"/>
       <c r="J51" s="2"/>
-      <c r="K51" s="3"/>
-      <c r="L51" s="3"/>
-      <c r="M51" s="3"/>
+      <c r="K51" s="49"/>
+      <c r="L51" s="49"/>
+      <c r="M51" s="49"/>
       <c r="N51" s="2"/>
       <c r="O51" s="2"/>
       <c r="P51" s="2"/>
@@ -3601,20 +3613,20 @@
       <c r="AP51" s="2"/>
       <c r="AQ51" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="18.75">
-      <c r="A52" s="3"/>
-      <c r="B52" s="3"/>
-      <c r="C52" s="3"/>
-      <c r="D52" s="3"/>
-      <c r="E52" s="3"/>
-      <c r="F52" s="3"/>
-      <c r="G52" s="3"/>
-      <c r="H52" s="3"/>
+    <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A52" s="49"/>
+      <c r="B52" s="49"/>
+      <c r="C52" s="49"/>
+      <c r="D52" s="49"/>
+      <c r="E52" s="49"/>
+      <c r="F52" s="49"/>
+      <c r="G52" s="49"/>
+      <c r="H52" s="49"/>
       <c r="I52" s="2"/>
       <c r="J52" s="2"/>
-      <c r="K52" s="3"/>
-      <c r="L52" s="3"/>
-      <c r="M52" s="3"/>
+      <c r="K52" s="49"/>
+      <c r="L52" s="49"/>
+      <c r="M52" s="49"/>
       <c r="N52" s="2"/>
       <c r="O52" s="2"/>
       <c r="P52" s="2"/>
@@ -3646,20 +3658,20 @@
       <c r="AP52" s="2"/>
       <c r="AQ52" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="18.75">
-      <c r="A53" s="3"/>
-      <c r="B53" s="3"/>
-      <c r="C53" s="3"/>
-      <c r="D53" s="3"/>
-      <c r="E53" s="3"/>
-      <c r="F53" s="3"/>
-      <c r="G53" s="3"/>
-      <c r="H53" s="3"/>
+    <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A53" s="49"/>
+      <c r="B53" s="49"/>
+      <c r="C53" s="49"/>
+      <c r="D53" s="49"/>
+      <c r="E53" s="49"/>
+      <c r="F53" s="49"/>
+      <c r="G53" s="49"/>
+      <c r="H53" s="49"/>
       <c r="I53" s="2"/>
       <c r="J53" s="2"/>
-      <c r="K53" s="3"/>
-      <c r="L53" s="3"/>
-      <c r="M53" s="3"/>
+      <c r="K53" s="49"/>
+      <c r="L53" s="49"/>
+      <c r="M53" s="49"/>
       <c r="N53" s="2"/>
       <c r="O53" s="2"/>
       <c r="P53" s="2"/>
@@ -3691,20 +3703,20 @@
       <c r="AP53" s="2"/>
       <c r="AQ53" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="54" customHeight="1" ht="18.75">
-      <c r="A54" s="3"/>
-      <c r="B54" s="3"/>
-      <c r="C54" s="3"/>
-      <c r="D54" s="3"/>
-      <c r="E54" s="3"/>
-      <c r="F54" s="3"/>
-      <c r="G54" s="3"/>
-      <c r="H54" s="3"/>
+    <row x14ac:dyDescent="0.25" r="54" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A54" s="49"/>
+      <c r="B54" s="49"/>
+      <c r="C54" s="49"/>
+      <c r="D54" s="49"/>
+      <c r="E54" s="49"/>
+      <c r="F54" s="49"/>
+      <c r="G54" s="49"/>
+      <c r="H54" s="49"/>
       <c r="I54" s="2"/>
       <c r="J54" s="2"/>
-      <c r="K54" s="3"/>
-      <c r="L54" s="3"/>
-      <c r="M54" s="3"/>
+      <c r="K54" s="49"/>
+      <c r="L54" s="49"/>
+      <c r="M54" s="49"/>
       <c r="N54" s="2"/>
       <c r="O54" s="2"/>
       <c r="P54" s="2"/>
@@ -3736,20 +3748,20 @@
       <c r="AP54" s="2"/>
       <c r="AQ54" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18.75">
-      <c r="A55" s="3"/>
-      <c r="B55" s="3"/>
-      <c r="C55" s="3"/>
-      <c r="D55" s="3"/>
-      <c r="E55" s="3"/>
-      <c r="F55" s="3"/>
-      <c r="G55" s="3"/>
-      <c r="H55" s="3"/>
+    <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A55" s="49"/>
+      <c r="B55" s="49"/>
+      <c r="C55" s="49"/>
+      <c r="D55" s="49"/>
+      <c r="E55" s="49"/>
+      <c r="F55" s="49"/>
+      <c r="G55" s="49"/>
+      <c r="H55" s="49"/>
       <c r="I55" s="2"/>
       <c r="J55" s="2"/>
-      <c r="K55" s="3"/>
-      <c r="L55" s="3"/>
-      <c r="M55" s="3"/>
+      <c r="K55" s="49"/>
+      <c r="L55" s="49"/>
+      <c r="M55" s="49"/>
       <c r="N55" s="2"/>
       <c r="O55" s="2"/>
       <c r="P55" s="2"/>
@@ -3781,20 +3793,20 @@
       <c r="AP55" s="2"/>
       <c r="AQ55" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="56" customHeight="1" ht="18.75">
-      <c r="A56" s="3"/>
-      <c r="B56" s="3"/>
-      <c r="C56" s="3"/>
-      <c r="D56" s="3"/>
-      <c r="E56" s="3"/>
-      <c r="F56" s="3"/>
-      <c r="G56" s="3"/>
-      <c r="H56" s="3"/>
+    <row x14ac:dyDescent="0.25" r="56" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A56" s="49"/>
+      <c r="B56" s="49"/>
+      <c r="C56" s="49"/>
+      <c r="D56" s="49"/>
+      <c r="E56" s="49"/>
+      <c r="F56" s="49"/>
+      <c r="G56" s="49"/>
+      <c r="H56" s="49"/>
       <c r="I56" s="2"/>
       <c r="J56" s="2"/>
-      <c r="K56" s="3"/>
-      <c r="L56" s="3"/>
-      <c r="M56" s="3"/>
+      <c r="K56" s="49"/>
+      <c r="L56" s="49"/>
+      <c r="M56" s="49"/>
       <c r="N56" s="2"/>
       <c r="O56" s="2"/>
       <c r="P56" s="2"/>
@@ -3826,20 +3838,20 @@
       <c r="AP56" s="2"/>
       <c r="AQ56" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="57" customHeight="1" ht="18.75">
-      <c r="A57" s="3"/>
-      <c r="B57" s="3"/>
-      <c r="C57" s="3"/>
-      <c r="D57" s="3"/>
-      <c r="E57" s="3"/>
-      <c r="F57" s="3"/>
-      <c r="G57" s="3"/>
-      <c r="H57" s="3"/>
+    <row x14ac:dyDescent="0.25" r="57" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A57" s="49"/>
+      <c r="B57" s="49"/>
+      <c r="C57" s="49"/>
+      <c r="D57" s="49"/>
+      <c r="E57" s="49"/>
+      <c r="F57" s="49"/>
+      <c r="G57" s="49"/>
+      <c r="H57" s="49"/>
       <c r="I57" s="2"/>
       <c r="J57" s="2"/>
-      <c r="K57" s="3"/>
-      <c r="L57" s="3"/>
-      <c r="M57" s="3"/>
+      <c r="K57" s="49"/>
+      <c r="L57" s="49"/>
+      <c r="M57" s="49"/>
       <c r="N57" s="2"/>
       <c r="O57" s="2"/>
       <c r="P57" s="2"/>
@@ -3871,20 +3883,20 @@
       <c r="AP57" s="2"/>
       <c r="AQ57" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="18.75">
-      <c r="A58" s="3"/>
-      <c r="B58" s="3"/>
-      <c r="C58" s="3"/>
-      <c r="D58" s="3"/>
-      <c r="E58" s="3"/>
-      <c r="F58" s="3"/>
-      <c r="G58" s="3"/>
-      <c r="H58" s="3"/>
+    <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A58" s="49"/>
+      <c r="B58" s="49"/>
+      <c r="C58" s="49"/>
+      <c r="D58" s="49"/>
+      <c r="E58" s="49"/>
+      <c r="F58" s="49"/>
+      <c r="G58" s="49"/>
+      <c r="H58" s="49"/>
       <c r="I58" s="2"/>
       <c r="J58" s="2"/>
-      <c r="K58" s="3"/>
-      <c r="L58" s="3"/>
-      <c r="M58" s="3"/>
+      <c r="K58" s="49"/>
+      <c r="L58" s="49"/>
+      <c r="M58" s="49"/>
       <c r="N58" s="2"/>
       <c r="O58" s="2"/>
       <c r="P58" s="2"/>
@@ -3916,20 +3928,20 @@
       <c r="AP58" s="2"/>
       <c r="AQ58" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="18.75">
-      <c r="A59" s="3"/>
-      <c r="B59" s="3"/>
-      <c r="C59" s="3"/>
-      <c r="D59" s="3"/>
-      <c r="E59" s="3"/>
-      <c r="F59" s="3"/>
-      <c r="G59" s="3"/>
-      <c r="H59" s="3"/>
+    <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A59" s="49"/>
+      <c r="B59" s="49"/>
+      <c r="C59" s="49"/>
+      <c r="D59" s="49"/>
+      <c r="E59" s="49"/>
+      <c r="F59" s="49"/>
+      <c r="G59" s="49"/>
+      <c r="H59" s="49"/>
       <c r="I59" s="2"/>
       <c r="J59" s="2"/>
-      <c r="K59" s="3"/>
-      <c r="L59" s="3"/>
-      <c r="M59" s="3"/>
+      <c r="K59" s="49"/>
+      <c r="L59" s="49"/>
+      <c r="M59" s="49"/>
       <c r="N59" s="2"/>
       <c r="O59" s="2"/>
       <c r="P59" s="2"/>
@@ -3961,20 +3973,20 @@
       <c r="AP59" s="2"/>
       <c r="AQ59" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="18.75">
-      <c r="A60" s="3"/>
-      <c r="B60" s="3"/>
-      <c r="C60" s="3"/>
-      <c r="D60" s="3"/>
-      <c r="E60" s="3"/>
-      <c r="F60" s="3"/>
-      <c r="G60" s="3"/>
-      <c r="H60" s="3"/>
+    <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A60" s="49"/>
+      <c r="B60" s="49"/>
+      <c r="C60" s="49"/>
+      <c r="D60" s="49"/>
+      <c r="E60" s="49"/>
+      <c r="F60" s="49"/>
+      <c r="G60" s="49"/>
+      <c r="H60" s="49"/>
       <c r="I60" s="2"/>
       <c r="J60" s="2"/>
-      <c r="K60" s="3"/>
-      <c r="L60" s="3"/>
-      <c r="M60" s="3"/>
+      <c r="K60" s="49"/>
+      <c r="L60" s="49"/>
+      <c r="M60" s="49"/>
       <c r="N60" s="2"/>
       <c r="O60" s="2"/>
       <c r="P60" s="2"/>
@@ -4006,20 +4018,20 @@
       <c r="AP60" s="2"/>
       <c r="AQ60" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="18.75">
-      <c r="A61" s="3"/>
-      <c r="B61" s="3"/>
-      <c r="C61" s="3"/>
-      <c r="D61" s="3"/>
-      <c r="E61" s="3"/>
-      <c r="F61" s="3"/>
-      <c r="G61" s="3"/>
-      <c r="H61" s="3"/>
+    <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A61" s="49"/>
+      <c r="B61" s="49"/>
+      <c r="C61" s="49"/>
+      <c r="D61" s="49"/>
+      <c r="E61" s="49"/>
+      <c r="F61" s="49"/>
+      <c r="G61" s="49"/>
+      <c r="H61" s="49"/>
       <c r="I61" s="2"/>
       <c r="J61" s="2"/>
-      <c r="K61" s="3"/>
-      <c r="L61" s="3"/>
-      <c r="M61" s="3"/>
+      <c r="K61" s="49"/>
+      <c r="L61" s="49"/>
+      <c r="M61" s="49"/>
       <c r="N61" s="2"/>
       <c r="O61" s="2"/>
       <c r="P61" s="2"/>
@@ -4051,20 +4063,20 @@
       <c r="AP61" s="2"/>
       <c r="AQ61" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="18.75">
-      <c r="A62" s="3"/>
-      <c r="B62" s="3"/>
-      <c r="C62" s="3"/>
-      <c r="D62" s="3"/>
-      <c r="E62" s="3"/>
-      <c r="F62" s="3"/>
-      <c r="G62" s="3"/>
-      <c r="H62" s="3"/>
+    <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A62" s="49"/>
+      <c r="B62" s="49"/>
+      <c r="C62" s="49"/>
+      <c r="D62" s="49"/>
+      <c r="E62" s="49"/>
+      <c r="F62" s="49"/>
+      <c r="G62" s="49"/>
+      <c r="H62" s="49"/>
       <c r="I62" s="2"/>
       <c r="J62" s="2"/>
-      <c r="K62" s="3"/>
-      <c r="L62" s="3"/>
-      <c r="M62" s="3"/>
+      <c r="K62" s="49"/>
+      <c r="L62" s="49"/>
+      <c r="M62" s="49"/>
       <c r="N62" s="2"/>
       <c r="O62" s="2"/>
       <c r="P62" s="2"/>
@@ -4096,20 +4108,20 @@
       <c r="AP62" s="2"/>
       <c r="AQ62" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="63" customHeight="1" ht="18.75">
-      <c r="A63" s="3"/>
-      <c r="B63" s="3"/>
-      <c r="C63" s="3"/>
-      <c r="D63" s="3"/>
-      <c r="E63" s="3"/>
-      <c r="F63" s="3"/>
-      <c r="G63" s="3"/>
-      <c r="H63" s="3"/>
+    <row x14ac:dyDescent="0.25" r="63" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A63" s="49"/>
+      <c r="B63" s="49"/>
+      <c r="C63" s="49"/>
+      <c r="D63" s="49"/>
+      <c r="E63" s="49"/>
+      <c r="F63" s="49"/>
+      <c r="G63" s="49"/>
+      <c r="H63" s="49"/>
       <c r="I63" s="2"/>
       <c r="J63" s="2"/>
-      <c r="K63" s="3"/>
-      <c r="L63" s="3"/>
-      <c r="M63" s="3"/>
+      <c r="K63" s="49"/>
+      <c r="L63" s="49"/>
+      <c r="M63" s="49"/>
       <c r="N63" s="2"/>
       <c r="O63" s="2"/>
       <c r="P63" s="2"/>
@@ -4141,20 +4153,20 @@
       <c r="AP63" s="2"/>
       <c r="AQ63" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="18.75">
-      <c r="A64" s="3"/>
-      <c r="B64" s="3"/>
-      <c r="C64" s="3"/>
-      <c r="D64" s="3"/>
-      <c r="E64" s="3"/>
-      <c r="F64" s="3"/>
-      <c r="G64" s="3"/>
-      <c r="H64" s="3"/>
+    <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A64" s="49"/>
+      <c r="B64" s="49"/>
+      <c r="C64" s="49"/>
+      <c r="D64" s="49"/>
+      <c r="E64" s="49"/>
+      <c r="F64" s="49"/>
+      <c r="G64" s="49"/>
+      <c r="H64" s="49"/>
       <c r="I64" s="2"/>
       <c r="J64" s="2"/>
-      <c r="K64" s="3"/>
-      <c r="L64" s="3"/>
-      <c r="M64" s="3"/>
+      <c r="K64" s="49"/>
+      <c r="L64" s="49"/>
+      <c r="M64" s="49"/>
       <c r="N64" s="2"/>
       <c r="O64" s="2"/>
       <c r="P64" s="2"/>
@@ -4186,20 +4198,20 @@
       <c r="AP64" s="2"/>
       <c r="AQ64" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="65" customHeight="1" ht="18.75">
-      <c r="A65" s="3"/>
-      <c r="B65" s="3"/>
-      <c r="C65" s="3"/>
-      <c r="D65" s="3"/>
-      <c r="E65" s="3"/>
-      <c r="F65" s="3"/>
-      <c r="G65" s="3"/>
-      <c r="H65" s="3"/>
+    <row x14ac:dyDescent="0.25" r="65" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A65" s="49"/>
+      <c r="B65" s="49"/>
+      <c r="C65" s="49"/>
+      <c r="D65" s="49"/>
+      <c r="E65" s="49"/>
+      <c r="F65" s="49"/>
+      <c r="G65" s="49"/>
+      <c r="H65" s="49"/>
       <c r="I65" s="2"/>
       <c r="J65" s="2"/>
-      <c r="K65" s="3"/>
-      <c r="L65" s="3"/>
-      <c r="M65" s="3"/>
+      <c r="K65" s="49"/>
+      <c r="L65" s="49"/>
+      <c r="M65" s="49"/>
       <c r="N65" s="2"/>
       <c r="O65" s="2"/>
       <c r="P65" s="2"/>
@@ -4231,20 +4243,20 @@
       <c r="AP65" s="2"/>
       <c r="AQ65" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="66" customHeight="1" ht="18.75">
-      <c r="A66" s="3"/>
-      <c r="B66" s="3"/>
-      <c r="C66" s="3"/>
-      <c r="D66" s="3"/>
-      <c r="E66" s="3"/>
-      <c r="F66" s="3"/>
-      <c r="G66" s="3"/>
-      <c r="H66" s="3"/>
+    <row x14ac:dyDescent="0.25" r="66" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A66" s="49"/>
+      <c r="B66" s="49"/>
+      <c r="C66" s="49"/>
+      <c r="D66" s="49"/>
+      <c r="E66" s="49"/>
+      <c r="F66" s="49"/>
+      <c r="G66" s="49"/>
+      <c r="H66" s="49"/>
       <c r="I66" s="2"/>
       <c r="J66" s="2"/>
-      <c r="K66" s="3"/>
-      <c r="L66" s="3"/>
-      <c r="M66" s="3"/>
+      <c r="K66" s="49"/>
+      <c r="L66" s="49"/>
+      <c r="M66" s="49"/>
       <c r="N66" s="2"/>
       <c r="O66" s="2"/>
       <c r="P66" s="2"/>
@@ -4276,20 +4288,20 @@
       <c r="AP66" s="2"/>
       <c r="AQ66" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="18.75">
-      <c r="A67" s="3"/>
-      <c r="B67" s="3"/>
-      <c r="C67" s="3"/>
-      <c r="D67" s="3"/>
-      <c r="E67" s="3"/>
-      <c r="F67" s="3"/>
-      <c r="G67" s="3"/>
-      <c r="H67" s="3"/>
+    <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A67" s="49"/>
+      <c r="B67" s="49"/>
+      <c r="C67" s="49"/>
+      <c r="D67" s="49"/>
+      <c r="E67" s="49"/>
+      <c r="F67" s="49"/>
+      <c r="G67" s="49"/>
+      <c r="H67" s="49"/>
       <c r="I67" s="2"/>
       <c r="J67" s="2"/>
-      <c r="K67" s="3"/>
-      <c r="L67" s="3"/>
-      <c r="M67" s="3"/>
+      <c r="K67" s="49"/>
+      <c r="L67" s="49"/>
+      <c r="M67" s="49"/>
       <c r="N67" s="2"/>
       <c r="O67" s="2"/>
       <c r="P67" s="2"/>
@@ -4321,20 +4333,20 @@
       <c r="AP67" s="2"/>
       <c r="AQ67" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="18.75">
-      <c r="A68" s="3"/>
-      <c r="B68" s="3"/>
-      <c r="C68" s="3"/>
-      <c r="D68" s="3"/>
-      <c r="E68" s="3"/>
-      <c r="F68" s="3"/>
-      <c r="G68" s="3"/>
-      <c r="H68" s="3"/>
+    <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A68" s="49"/>
+      <c r="B68" s="49"/>
+      <c r="C68" s="49"/>
+      <c r="D68" s="49"/>
+      <c r="E68" s="49"/>
+      <c r="F68" s="49"/>
+      <c r="G68" s="49"/>
+      <c r="H68" s="49"/>
       <c r="I68" s="2"/>
       <c r="J68" s="2"/>
-      <c r="K68" s="3"/>
-      <c r="L68" s="3"/>
-      <c r="M68" s="3"/>
+      <c r="K68" s="49"/>
+      <c r="L68" s="49"/>
+      <c r="M68" s="49"/>
       <c r="N68" s="2"/>
       <c r="O68" s="2"/>
       <c r="P68" s="2"/>
@@ -4366,20 +4378,20 @@
       <c r="AP68" s="2"/>
       <c r="AQ68" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="18.75">
-      <c r="A69" s="3"/>
-      <c r="B69" s="3"/>
-      <c r="C69" s="3"/>
-      <c r="D69" s="3"/>
-      <c r="E69" s="3"/>
-      <c r="F69" s="3"/>
-      <c r="G69" s="3"/>
-      <c r="H69" s="3"/>
+    <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A69" s="49"/>
+      <c r="B69" s="49"/>
+      <c r="C69" s="49"/>
+      <c r="D69" s="49"/>
+      <c r="E69" s="49"/>
+      <c r="F69" s="49"/>
+      <c r="G69" s="49"/>
+      <c r="H69" s="49"/>
       <c r="I69" s="2"/>
       <c r="J69" s="2"/>
-      <c r="K69" s="3"/>
-      <c r="L69" s="3"/>
-      <c r="M69" s="3"/>
+      <c r="K69" s="49"/>
+      <c r="L69" s="49"/>
+      <c r="M69" s="49"/>
       <c r="N69" s="2"/>
       <c r="O69" s="2"/>
       <c r="P69" s="2"/>
@@ -4411,20 +4423,20 @@
       <c r="AP69" s="2"/>
       <c r="AQ69" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="18.75">
-      <c r="A70" s="3"/>
-      <c r="B70" s="3"/>
-      <c r="C70" s="3"/>
-      <c r="D70" s="3"/>
-      <c r="E70" s="3"/>
-      <c r="F70" s="3"/>
-      <c r="G70" s="3"/>
-      <c r="H70" s="3"/>
+    <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A70" s="49"/>
+      <c r="B70" s="49"/>
+      <c r="C70" s="49"/>
+      <c r="D70" s="49"/>
+      <c r="E70" s="49"/>
+      <c r="F70" s="49"/>
+      <c r="G70" s="49"/>
+      <c r="H70" s="49"/>
       <c r="I70" s="2"/>
       <c r="J70" s="2"/>
-      <c r="K70" s="3"/>
-      <c r="L70" s="3"/>
-      <c r="M70" s="3"/>
+      <c r="K70" s="49"/>
+      <c r="L70" s="49"/>
+      <c r="M70" s="49"/>
       <c r="N70" s="2"/>
       <c r="O70" s="2"/>
       <c r="P70" s="2"/>
@@ -4456,20 +4468,20 @@
       <c r="AP70" s="2"/>
       <c r="AQ70" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="71" customHeight="1" ht="18.75">
-      <c r="A71" s="3"/>
-      <c r="B71" s="3"/>
-      <c r="C71" s="3"/>
-      <c r="D71" s="3"/>
-      <c r="E71" s="3"/>
-      <c r="F71" s="3"/>
-      <c r="G71" s="3"/>
-      <c r="H71" s="3"/>
+    <row x14ac:dyDescent="0.25" r="71" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A71" s="49"/>
+      <c r="B71" s="49"/>
+      <c r="C71" s="49"/>
+      <c r="D71" s="49"/>
+      <c r="E71" s="49"/>
+      <c r="F71" s="49"/>
+      <c r="G71" s="49"/>
+      <c r="H71" s="49"/>
       <c r="I71" s="2"/>
       <c r="J71" s="2"/>
-      <c r="K71" s="3"/>
-      <c r="L71" s="3"/>
-      <c r="M71" s="3"/>
+      <c r="K71" s="49"/>
+      <c r="L71" s="49"/>
+      <c r="M71" s="49"/>
       <c r="N71" s="2"/>
       <c r="O71" s="2"/>
       <c r="P71" s="2"/>
@@ -4501,20 +4513,20 @@
       <c r="AP71" s="2"/>
       <c r="AQ71" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="72" customHeight="1" ht="18.75">
-      <c r="A72" s="3"/>
-      <c r="B72" s="3"/>
-      <c r="C72" s="3"/>
-      <c r="D72" s="3"/>
-      <c r="E72" s="3"/>
-      <c r="F72" s="3"/>
-      <c r="G72" s="3"/>
-      <c r="H72" s="3"/>
+    <row x14ac:dyDescent="0.25" r="72" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A72" s="49"/>
+      <c r="B72" s="49"/>
+      <c r="C72" s="49"/>
+      <c r="D72" s="49"/>
+      <c r="E72" s="49"/>
+      <c r="F72" s="49"/>
+      <c r="G72" s="49"/>
+      <c r="H72" s="49"/>
       <c r="I72" s="2"/>
       <c r="J72" s="2"/>
-      <c r="K72" s="3"/>
-      <c r="L72" s="3"/>
-      <c r="M72" s="3"/>
+      <c r="K72" s="49"/>
+      <c r="L72" s="49"/>
+      <c r="M72" s="49"/>
       <c r="N72" s="2"/>
       <c r="O72" s="2"/>
       <c r="P72" s="2"/>
@@ -4546,20 +4558,20 @@
       <c r="AP72" s="2"/>
       <c r="AQ72" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="73" customHeight="1" ht="18.75">
-      <c r="A73" s="3"/>
-      <c r="B73" s="3"/>
-      <c r="C73" s="3"/>
-      <c r="D73" s="3"/>
-      <c r="E73" s="3"/>
-      <c r="F73" s="3"/>
-      <c r="G73" s="3"/>
-      <c r="H73" s="3"/>
+    <row x14ac:dyDescent="0.25" r="73" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A73" s="49"/>
+      <c r="B73" s="49"/>
+      <c r="C73" s="49"/>
+      <c r="D73" s="49"/>
+      <c r="E73" s="49"/>
+      <c r="F73" s="49"/>
+      <c r="G73" s="49"/>
+      <c r="H73" s="49"/>
       <c r="I73" s="2"/>
       <c r="J73" s="2"/>
-      <c r="K73" s="3"/>
-      <c r="L73" s="3"/>
-      <c r="M73" s="3"/>
+      <c r="K73" s="49"/>
+      <c r="L73" s="49"/>
+      <c r="M73" s="49"/>
       <c r="N73" s="2"/>
       <c r="O73" s="2"/>
       <c r="P73" s="2"/>
@@ -4591,20 +4603,20 @@
       <c r="AP73" s="2"/>
       <c r="AQ73" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="74" customHeight="1" ht="18.75">
-      <c r="A74" s="3"/>
-      <c r="B74" s="3"/>
-      <c r="C74" s="3"/>
-      <c r="D74" s="3"/>
-      <c r="E74" s="3"/>
-      <c r="F74" s="3"/>
-      <c r="G74" s="3"/>
-      <c r="H74" s="3"/>
+    <row x14ac:dyDescent="0.25" r="74" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A74" s="49"/>
+      <c r="B74" s="49"/>
+      <c r="C74" s="49"/>
+      <c r="D74" s="49"/>
+      <c r="E74" s="49"/>
+      <c r="F74" s="49"/>
+      <c r="G74" s="49"/>
+      <c r="H74" s="49"/>
       <c r="I74" s="2"/>
       <c r="J74" s="2"/>
-      <c r="K74" s="3"/>
-      <c r="L74" s="3"/>
-      <c r="M74" s="3"/>
+      <c r="K74" s="49"/>
+      <c r="L74" s="49"/>
+      <c r="M74" s="49"/>
       <c r="N74" s="2"/>
       <c r="O74" s="2"/>
       <c r="P74" s="2"/>
@@ -4636,20 +4648,20 @@
       <c r="AP74" s="2"/>
       <c r="AQ74" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="75" customHeight="1" ht="18.75">
-      <c r="A75" s="3"/>
-      <c r="B75" s="3"/>
-      <c r="C75" s="3"/>
-      <c r="D75" s="3"/>
-      <c r="E75" s="3"/>
-      <c r="F75" s="3"/>
-      <c r="G75" s="3"/>
-      <c r="H75" s="3"/>
+    <row x14ac:dyDescent="0.25" r="75" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A75" s="49"/>
+      <c r="B75" s="49"/>
+      <c r="C75" s="49"/>
+      <c r="D75" s="49"/>
+      <c r="E75" s="49"/>
+      <c r="F75" s="49"/>
+      <c r="G75" s="49"/>
+      <c r="H75" s="49"/>
       <c r="I75" s="2"/>
       <c r="J75" s="2"/>
-      <c r="K75" s="3"/>
-      <c r="L75" s="3"/>
-      <c r="M75" s="3"/>
+      <c r="K75" s="49"/>
+      <c r="L75" s="49"/>
+      <c r="M75" s="49"/>
       <c r="N75" s="2"/>
       <c r="O75" s="2"/>
       <c r="P75" s="2"/>
@@ -4681,20 +4693,20 @@
       <c r="AP75" s="2"/>
       <c r="AQ75" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="76" customHeight="1" ht="18.75">
-      <c r="A76" s="3"/>
-      <c r="B76" s="3"/>
-      <c r="C76" s="3"/>
-      <c r="D76" s="3"/>
-      <c r="E76" s="3"/>
-      <c r="F76" s="3"/>
-      <c r="G76" s="3"/>
-      <c r="H76" s="3"/>
+    <row x14ac:dyDescent="0.25" r="76" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A76" s="49"/>
+      <c r="B76" s="49"/>
+      <c r="C76" s="49"/>
+      <c r="D76" s="49"/>
+      <c r="E76" s="49"/>
+      <c r="F76" s="49"/>
+      <c r="G76" s="49"/>
+      <c r="H76" s="49"/>
       <c r="I76" s="2"/>
       <c r="J76" s="2"/>
-      <c r="K76" s="3"/>
-      <c r="L76" s="3"/>
-      <c r="M76" s="3"/>
+      <c r="K76" s="49"/>
+      <c r="L76" s="49"/>
+      <c r="M76" s="49"/>
       <c r="N76" s="2"/>
       <c r="O76" s="2"/>
       <c r="P76" s="2"/>
@@ -4726,20 +4738,20 @@
       <c r="AP76" s="2"/>
       <c r="AQ76" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="77" customHeight="1" ht="18.75">
-      <c r="A77" s="3"/>
-      <c r="B77" s="3"/>
-      <c r="C77" s="3"/>
-      <c r="D77" s="3"/>
-      <c r="E77" s="3"/>
-      <c r="F77" s="3"/>
-      <c r="G77" s="3"/>
-      <c r="H77" s="3"/>
+    <row x14ac:dyDescent="0.25" r="77" customHeight="1" ht="18.75" customFormat="1" s="19">
+      <c r="A77" s="49"/>
+      <c r="B77" s="49"/>
+      <c r="C77" s="49"/>
+      <c r="D77" s="49"/>
+      <c r="E77" s="49"/>
+      <c r="F77" s="49"/>
+      <c r="G77" s="49"/>
+      <c r="H77" s="49"/>
       <c r="I77" s="2"/>
       <c r="J77" s="2"/>
-      <c r="K77" s="3"/>
-      <c r="L77" s="3"/>
-      <c r="M77" s="3"/>
+      <c r="K77" s="49"/>
+      <c r="L77" s="49"/>
+      <c r="M77" s="49"/>
       <c r="N77" s="2"/>
       <c r="O77" s="2"/>
       <c r="P77" s="2"/>

</xml_diff>